<commit_message>
Atualização automática: reparaveis_rma (24/08/2026 18:39)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -3809,16 +3809,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -3834,7 +3826,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -3842,30 +3834,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -4165,52 +4139,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -4224,7 +4198,7 @@
       <c r="C2">
         <v>2026</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="1">
         <v>45972</v>
       </c>
       <c r="F2" t="s">
@@ -4265,7 +4239,7 @@
       <c r="C3">
         <v>2026</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
         <v>46014</v>
       </c>
       <c r="F3" t="s">
@@ -4306,7 +4280,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45916</v>
       </c>
       <c r="F4" t="s">
@@ -4347,7 +4321,7 @@
       <c r="C5">
         <v>2026</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="1">
         <v>45897</v>
       </c>
       <c r="H5" t="s">
@@ -4382,7 +4356,7 @@
       <c r="C6">
         <v>2026</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>45916</v>
       </c>
       <c r="F6" t="s">
@@ -4423,7 +4397,7 @@
       <c r="C7">
         <v>2026</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="1">
         <v>46086</v>
       </c>
       <c r="G7" t="s">
@@ -4461,7 +4435,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>45869</v>
       </c>
       <c r="F8" t="s">
@@ -4502,7 +4476,7 @@
       <c r="C9">
         <v>2026</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="1">
         <v>45877</v>
       </c>
       <c r="F9" t="s">
@@ -4543,7 +4517,7 @@
       <c r="C10">
         <v>2026</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="1">
         <v>46086</v>
       </c>
       <c r="G10" t="s">
@@ -4581,7 +4555,7 @@
       <c r="C11">
         <v>2026</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
         <v>45863</v>
       </c>
       <c r="F11" t="s">
@@ -4622,7 +4596,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45863</v>
       </c>
       <c r="F12" t="s">
@@ -4663,7 +4637,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45873</v>
       </c>
       <c r="F13" t="s">
@@ -4704,7 +4678,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>46086</v>
       </c>
       <c r="F14" t="s">
@@ -4745,7 +4719,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -4783,7 +4757,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45838</v>
       </c>
       <c r="F16" t="s">
@@ -4824,7 +4798,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45800</v>
       </c>
       <c r="F17" t="s">
@@ -4865,7 +4839,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>45849</v>
       </c>
       <c r="F18" t="s">
@@ -4906,7 +4880,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45838</v>
       </c>
       <c r="F19" t="s">
@@ -4947,7 +4921,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45915</v>
       </c>
       <c r="F20" t="s">
@@ -4988,7 +4962,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45849</v>
       </c>
       <c r="F21" t="s">
@@ -5029,7 +5003,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>45800</v>
       </c>
       <c r="F22" t="s">
@@ -5070,7 +5044,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46119</v>
       </c>
       <c r="F23" t="s">
@@ -5111,7 +5085,7 @@
       <c r="C24">
         <v>2026</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="1">
         <v>45854</v>
       </c>
       <c r="F24" t="s">
@@ -5152,7 +5126,7 @@
       <c r="C25">
         <v>2026</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D25" s="1">
         <v>45849</v>
       </c>
       <c r="F25" t="s">
@@ -5193,7 +5167,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>46119</v>
       </c>
       <c r="F26" t="s">
@@ -5234,7 +5208,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>46092</v>
       </c>
       <c r="F27" t="s">
@@ -5275,7 +5249,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>46122</v>
       </c>
       <c r="F28" t="s">
@@ -5316,7 +5290,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>46122</v>
       </c>
       <c r="F29" t="s">
@@ -5357,7 +5331,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>46135</v>
       </c>
       <c r="F30" t="s">
@@ -5398,7 +5372,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>46086</v>
       </c>
       <c r="F31" t="s">
@@ -5439,7 +5413,7 @@
       <c r="C32">
         <v>2026</v>
       </c>
-      <c r="D32" s="2">
+      <c r="D32" s="1">
         <v>46104</v>
       </c>
       <c r="F32" t="s">
@@ -5480,7 +5454,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45972</v>
       </c>
       <c r="G33" t="s">
@@ -5518,7 +5492,7 @@
       <c r="C34">
         <v>2026</v>
       </c>
-      <c r="D34" s="2">
+      <c r="D34" s="1">
         <v>45810</v>
       </c>
       <c r="F34" t="s">
@@ -5559,7 +5533,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>45937</v>
       </c>
       <c r="F35" t="s">
@@ -5600,7 +5574,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45937</v>
       </c>
       <c r="F36" t="s">
@@ -5641,7 +5615,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45845</v>
       </c>
       <c r="F37" t="s">
@@ -5682,7 +5656,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46077</v>
       </c>
       <c r="F38" t="s">
@@ -5723,7 +5697,7 @@
       <c r="C39">
         <v>2026</v>
       </c>
-      <c r="D39" s="2">
+      <c r="D39" s="1">
         <v>45971</v>
       </c>
       <c r="F39" t="s">
@@ -5764,7 +5738,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>45817</v>
       </c>
       <c r="F40" t="s">
@@ -5805,7 +5779,7 @@
       <c r="C41">
         <v>2026</v>
       </c>
-      <c r="D41" s="2">
+      <c r="D41" s="1">
         <v>45965</v>
       </c>
       <c r="G41" t="s">
@@ -5843,7 +5817,7 @@
       <c r="C42">
         <v>2026</v>
       </c>
-      <c r="D42" s="2">
+      <c r="D42" s="1">
         <v>46072</v>
       </c>
       <c r="F42" t="s">
@@ -5884,7 +5858,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46072</v>
       </c>
       <c r="H43" t="s">
@@ -5919,7 +5893,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>45804</v>
       </c>
       <c r="F44" t="s">
@@ -5960,7 +5934,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>45804</v>
       </c>
       <c r="F45" t="s">
@@ -6001,7 +5975,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>45804</v>
       </c>
       <c r="F46" t="s">
@@ -6042,7 +6016,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>45804</v>
       </c>
       <c r="F47" t="s">
@@ -6083,7 +6057,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45804</v>
       </c>
       <c r="F48" t="s">
@@ -6124,7 +6098,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45804</v>
       </c>
       <c r="F49" t="s">
@@ -6165,7 +6139,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45821</v>
       </c>
       <c r="F50" t="s">
@@ -6206,7 +6180,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45821</v>
       </c>
       <c r="H51" t="s">
@@ -6241,7 +6215,7 @@
       <c r="C52">
         <v>2026</v>
       </c>
-      <c r="D52" s="2">
+      <c r="D52" s="1">
         <v>45891</v>
       </c>
       <c r="F52" t="s">
@@ -6282,7 +6256,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45817</v>
       </c>
       <c r="G53" t="s">
@@ -6320,7 +6294,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>45883</v>
       </c>
       <c r="G54" t="s">
@@ -6358,7 +6332,7 @@
       <c r="C55">
         <v>2026</v>
       </c>
-      <c r="D55" s="2">
+      <c r="D55" s="1">
         <v>45817</v>
       </c>
       <c r="G55" t="s">
@@ -6396,7 +6370,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45883</v>
       </c>
       <c r="G56" t="s">
@@ -6434,7 +6408,7 @@
       <c r="C57">
         <v>2026</v>
       </c>
-      <c r="D57" s="2">
+      <c r="D57" s="1">
         <v>45971</v>
       </c>
       <c r="F57" t="s">
@@ -6475,7 +6449,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45849</v>
       </c>
       <c r="F58" t="s">
@@ -6516,7 +6490,7 @@
       <c r="C59">
         <v>2026</v>
       </c>
-      <c r="D59" s="2">
+      <c r="D59" s="1">
         <v>45849</v>
       </c>
       <c r="F59" t="s">
@@ -6557,7 +6531,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45863</v>
       </c>
       <c r="F60" t="s">
@@ -6598,7 +6572,7 @@
       <c r="C61">
         <v>2026</v>
       </c>
-      <c r="D61" s="2">
+      <c r="D61" s="1">
         <v>45810</v>
       </c>
       <c r="F61" t="s">
@@ -6639,7 +6613,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>45926</v>
       </c>
       <c r="F62" t="s">
@@ -6680,7 +6654,7 @@
       <c r="C63">
         <v>2026</v>
       </c>
-      <c r="D63" s="2">
+      <c r="D63" s="1">
         <v>45971</v>
       </c>
       <c r="F63" t="s">
@@ -6721,7 +6695,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46164</v>
       </c>
       <c r="F64" t="s">
@@ -6762,7 +6736,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45986</v>
       </c>
       <c r="G65" t="s">
@@ -6841,7 +6815,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45786</v>
       </c>
       <c r="F67" t="s">
@@ -6882,7 +6856,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45777</v>
       </c>
       <c r="F68" t="s">
@@ -6923,7 +6897,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45869</v>
       </c>
       <c r="F69" t="s">
@@ -6964,7 +6938,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45891</v>
       </c>
       <c r="F70" t="s">
@@ -7005,7 +6979,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45863</v>
       </c>
       <c r="F71" t="s">
@@ -7046,7 +7020,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45769</v>
       </c>
       <c r="F72" t="s">
@@ -7087,7 +7061,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45769</v>
       </c>
       <c r="F73" t="s">
@@ -7128,7 +7102,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45894</v>
       </c>
       <c r="F74" t="s">
@@ -7169,7 +7143,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45894</v>
       </c>
       <c r="F75" t="s">
@@ -7210,7 +7184,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45971</v>
       </c>
       <c r="F76" t="s">
@@ -7251,7 +7225,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45971</v>
       </c>
       <c r="F77" t="s">
@@ -7292,7 +7266,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -7333,7 +7307,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45996</v>
       </c>
       <c r="G79" t="s">
@@ -7371,7 +7345,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45986</v>
       </c>
       <c r="G80" t="s">
@@ -7409,7 +7383,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45769</v>
       </c>
       <c r="F81" t="s">
@@ -7450,7 +7424,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45769</v>
       </c>
       <c r="F82" t="s">
@@ -7491,7 +7465,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45849</v>
       </c>
       <c r="F83" t="s">
@@ -7532,7 +7506,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45849</v>
       </c>
       <c r="G84" t="s">
@@ -7570,7 +7544,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>45891</v>
       </c>
       <c r="F85" t="s">
@@ -7611,7 +7585,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45769</v>
       </c>
       <c r="F86" t="s">
@@ -7652,7 +7626,7 @@
       <c r="C87">
         <v>2026</v>
       </c>
-      <c r="D87" s="2">
+      <c r="D87" s="1">
         <v>45889</v>
       </c>
       <c r="F87" t="s">
@@ -7693,7 +7667,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45945</v>
       </c>
       <c r="G88" t="s">
@@ -7731,7 +7705,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45945</v>
       </c>
       <c r="G89" t="s">
@@ -7769,7 +7743,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>46119</v>
       </c>
       <c r="F90" t="s">
@@ -7810,7 +7784,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>46029</v>
       </c>
       <c r="F91" t="s">
@@ -7851,7 +7825,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>46029</v>
       </c>
       <c r="F92" t="s">
@@ -7892,7 +7866,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>46119</v>
       </c>
       <c r="F93" t="s">
@@ -7933,7 +7907,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>46230</v>
       </c>
       <c r="F94" t="s">
@@ -7974,7 +7948,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>46119</v>
       </c>
       <c r="F95" t="s">
@@ -8015,7 +7989,7 @@
       <c r="C96">
         <v>2026</v>
       </c>
-      <c r="D96" s="2">
+      <c r="D96" s="1">
         <v>46119</v>
       </c>
       <c r="F96" t="s">
@@ -8056,7 +8030,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45931</v>
       </c>
       <c r="F97" t="s">
@@ -8097,7 +8071,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45894</v>
       </c>
       <c r="G98" t="s">
@@ -8135,7 +8109,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>46119</v>
       </c>
       <c r="F99" t="s">
@@ -8176,7 +8150,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45889</v>
       </c>
       <c r="F100" t="s">
@@ -8217,7 +8191,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45876</v>
       </c>
       <c r="G101" t="s">
@@ -8255,7 +8229,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45876</v>
       </c>
       <c r="F102" t="s">
@@ -8296,7 +8270,7 @@
       <c r="C103">
         <v>2026</v>
       </c>
-      <c r="D103" s="2">
+      <c r="D103" s="1">
         <v>46230</v>
       </c>
       <c r="F103" t="s">
@@ -8337,7 +8311,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45889</v>
       </c>
       <c r="F104" t="s">
@@ -8378,7 +8352,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>46230</v>
       </c>
       <c r="F105" t="s">
@@ -8419,7 +8393,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>46140</v>
       </c>
       <c r="F106" t="s">
@@ -8460,7 +8434,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45889</v>
       </c>
       <c r="F107" t="s">
@@ -8501,7 +8475,7 @@
       <c r="C108">
         <v>2026</v>
       </c>
-      <c r="D108" s="2">
+      <c r="D108" s="1">
         <v>45952</v>
       </c>
       <c r="F108" t="s">
@@ -8539,7 +8513,7 @@
       <c r="C109">
         <v>2026</v>
       </c>
-      <c r="D109" s="2">
+      <c r="D109" s="1">
         <v>46230</v>
       </c>
       <c r="F109" t="s">
@@ -8580,7 +8554,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>46029</v>
       </c>
       <c r="G110" t="s">
@@ -8618,7 +8592,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>46029</v>
       </c>
       <c r="G111" t="s">
@@ -8656,7 +8630,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>46119</v>
       </c>
       <c r="F112" t="s">
@@ -8697,7 +8671,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>46140</v>
       </c>
       <c r="F113" t="s">
@@ -8738,7 +8712,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>46230</v>
       </c>
       <c r="F114" t="s">
@@ -8779,7 +8753,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46230</v>
       </c>
       <c r="F115" t="s">
@@ -8820,7 +8794,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46119</v>
       </c>
       <c r="F116" t="s">
@@ -8861,7 +8835,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46230</v>
       </c>
       <c r="F117" t="s">
@@ -8902,7 +8876,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46140</v>
       </c>
       <c r="F118" t="s">
@@ -8943,7 +8917,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>45876</v>
       </c>
       <c r="F119" t="s">
@@ -8984,7 +8958,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>45863</v>
       </c>
       <c r="F120" t="s">
@@ -9025,7 +8999,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>45863</v>
       </c>
       <c r="F121" t="s">
@@ -9066,7 +9040,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45863</v>
       </c>
       <c r="F122" t="s">
@@ -9107,7 +9081,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45860</v>
       </c>
       <c r="F123" t="s">
@@ -9148,7 +9122,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -9189,7 +9163,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45814</v>
       </c>
       <c r="F125" t="s">
@@ -9230,7 +9204,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45817</v>
       </c>
       <c r="F126" t="s">
@@ -9271,7 +9245,7 @@
       <c r="C127">
         <v>2026</v>
       </c>
-      <c r="D127" s="2">
+      <c r="D127" s="1">
         <v>45971</v>
       </c>
       <c r="F127" t="s">
@@ -9312,7 +9286,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45971</v>
       </c>
       <c r="F128" t="s">
@@ -9353,7 +9327,7 @@
       <c r="C129">
         <v>2026</v>
       </c>
-      <c r="D129" s="2">
+      <c r="D129" s="1">
         <v>45860</v>
       </c>
       <c r="G129" t="s">
@@ -9391,7 +9365,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>45856</v>
       </c>
       <c r="F130" t="s">
@@ -9432,7 +9406,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>46064</v>
       </c>
       <c r="F131" t="s">
@@ -9473,7 +9447,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>45982</v>
       </c>
       <c r="G132" t="s">
@@ -9511,7 +9485,7 @@
       <c r="C133">
         <v>2026</v>
       </c>
-      <c r="D133" s="2">
+      <c r="D133" s="1">
         <v>46157</v>
       </c>
       <c r="H133" t="s">
@@ -9546,7 +9520,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>45762</v>
       </c>
       <c r="F134" t="s">
@@ -9587,7 +9561,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45816</v>
       </c>
       <c r="F135" t="s">
@@ -9628,7 +9602,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45816</v>
       </c>
       <c r="F136" t="s">
@@ -9707,7 +9681,7 @@
       <c r="C138">
         <v>2026</v>
       </c>
-      <c r="D138" s="2">
+      <c r="D138" s="1">
         <v>46101</v>
       </c>
       <c r="F138" t="s">
@@ -9748,7 +9722,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46101</v>
       </c>
       <c r="F139" t="s">
@@ -9789,7 +9763,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46105</v>
       </c>
       <c r="F140" t="s">
@@ -9830,7 +9804,7 @@
       <c r="C141">
         <v>2026</v>
       </c>
-      <c r="D141" s="2">
+      <c r="D141" s="1">
         <v>45889</v>
       </c>
       <c r="F141" t="s">
@@ -9871,7 +9845,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>45814</v>
       </c>
       <c r="F142" t="s">
@@ -9912,7 +9886,7 @@
       <c r="C143">
         <v>2026</v>
       </c>
-      <c r="D143" s="2">
+      <c r="D143" s="1">
         <v>45889</v>
       </c>
       <c r="F143" t="s">
@@ -9953,7 +9927,7 @@
       <c r="C144">
         <v>2026</v>
       </c>
-      <c r="D144" s="2">
+      <c r="D144" s="1">
         <v>45814</v>
       </c>
       <c r="F144" t="s">
@@ -9994,7 +9968,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>45889</v>
       </c>
       <c r="F145" t="s">
@@ -10035,7 +10009,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46139</v>
       </c>
       <c r="H146" t="s">
@@ -10070,7 +10044,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>45889</v>
       </c>
       <c r="F147" t="s">
@@ -10111,7 +10085,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>45814</v>
       </c>
       <c r="F148" t="s">
@@ -10152,7 +10126,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>45889</v>
       </c>
       <c r="F149" t="s">
@@ -10193,7 +10167,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>45931</v>
       </c>
       <c r="F150" t="s">
@@ -10234,7 +10208,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45889</v>
       </c>
       <c r="F151" t="s">
@@ -10275,7 +10249,7 @@
       <c r="C152">
         <v>2026</v>
       </c>
-      <c r="D152" s="2">
+      <c r="D152" s="1">
         <v>45876</v>
       </c>
       <c r="F152" t="s">
@@ -10316,7 +10290,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45876</v>
       </c>
       <c r="F153" t="s">
@@ -10357,7 +10331,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45876</v>
       </c>
       <c r="F154" t="s">
@@ -10398,7 +10372,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>46119</v>
       </c>
       <c r="F155" t="s">
@@ -10439,7 +10413,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>46119</v>
       </c>
       <c r="F156" t="s">
@@ -10480,7 +10454,7 @@
       <c r="C157">
         <v>2026</v>
       </c>
-      <c r="D157" s="2">
+      <c r="D157" s="1">
         <v>45961</v>
       </c>
       <c r="F157" t="s">
@@ -10521,7 +10495,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>45860</v>
       </c>
       <c r="F158" t="s">
@@ -10562,7 +10536,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45993</v>
       </c>
       <c r="G159" t="s">
@@ -10600,7 +10574,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45853</v>
       </c>
       <c r="F160" t="s">
@@ -10641,7 +10615,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>46119</v>
       </c>
       <c r="F161" t="s">
@@ -10720,7 +10694,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>46191</v>
       </c>
       <c r="F163" t="s">
@@ -10761,7 +10735,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>46191</v>
       </c>
       <c r="F164" t="s">
@@ -10802,7 +10776,7 @@
       <c r="C165">
         <v>2026</v>
       </c>
-      <c r="D165" s="2">
+      <c r="D165" s="1">
         <v>46191</v>
       </c>
       <c r="F165" t="s">
@@ -10843,7 +10817,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>45932</v>
       </c>
       <c r="G166" t="s">
@@ -10881,7 +10855,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>46191</v>
       </c>
       <c r="F167" t="s">
@@ -10922,7 +10896,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46119</v>
       </c>
       <c r="F168" t="s">
@@ -10963,7 +10937,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45946</v>
       </c>
       <c r="G169" t="s">
@@ -11001,7 +10975,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45937</v>
       </c>
       <c r="F170" t="s">
@@ -11042,7 +11016,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45849</v>
       </c>
       <c r="F171" t="s">
@@ -11083,7 +11057,7 @@
       <c r="C172">
         <v>2026</v>
       </c>
-      <c r="D172" s="2">
+      <c r="D172" s="1">
         <v>45876</v>
       </c>
       <c r="F172" t="s">
@@ -11124,7 +11098,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46008</v>
       </c>
       <c r="F173" t="s">
@@ -11206,7 +11180,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>45973</v>
       </c>
       <c r="F175" t="s">
@@ -11247,7 +11221,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>46014</v>
       </c>
       <c r="F176" t="s">
@@ -11288,7 +11262,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45876</v>
       </c>
       <c r="F177" t="s">
@@ -11329,7 +11303,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45937</v>
       </c>
       <c r="F178" t="s">
@@ -11370,7 +11344,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45980</v>
       </c>
       <c r="F179" t="s">
@@ -11411,7 +11385,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45979</v>
       </c>
       <c r="F180" t="s">
@@ -11452,7 +11426,7 @@
       <c r="C181">
         <v>2026</v>
       </c>
-      <c r="D181" s="2">
+      <c r="D181" s="1">
         <v>45979</v>
       </c>
       <c r="F181" t="s">
@@ -11493,7 +11467,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>45979</v>
       </c>
       <c r="F182" t="s">
@@ -11534,7 +11508,7 @@
       <c r="C183">
         <v>2026</v>
       </c>
-      <c r="D183" s="2">
+      <c r="D183" s="1">
         <v>45971</v>
       </c>
       <c r="F183" t="s">
@@ -11575,7 +11549,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45971</v>
       </c>
       <c r="F184" t="s">
@@ -11616,7 +11590,7 @@
       <c r="C185">
         <v>2026</v>
       </c>
-      <c r="D185" s="2">
+      <c r="D185" s="1">
         <v>45971</v>
       </c>
       <c r="F185" t="s">
@@ -11657,7 +11631,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45889</v>
       </c>
       <c r="F186" t="s">
@@ -11698,7 +11672,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45859</v>
       </c>
       <c r="F187" t="s">
@@ -11739,7 +11713,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45918</v>
       </c>
       <c r="F188" t="s">
@@ -11780,7 +11754,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45874</v>
       </c>
       <c r="F189" t="s">
@@ -11821,7 +11795,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45975</v>
       </c>
       <c r="F190" t="s">
@@ -11859,7 +11833,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45975</v>
       </c>
       <c r="F191" t="s">
@@ -11897,7 +11871,7 @@
       <c r="C192">
         <v>2026</v>
       </c>
-      <c r="D192" s="2">
+      <c r="D192" s="1">
         <v>45975</v>
       </c>
       <c r="F192" t="s">
@@ -11935,7 +11909,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>46119</v>
       </c>
       <c r="F193" t="s">
@@ -11976,7 +11950,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>45802</v>
       </c>
       <c r="F194" t="s">
@@ -12017,7 +11991,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>45804</v>
       </c>
       <c r="F195" t="s">
@@ -12058,7 +12032,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>46097</v>
       </c>
       <c r="F196" t="s">
@@ -12099,7 +12073,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="G197" t="s">
@@ -12137,7 +12111,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45889</v>
       </c>
       <c r="F198" t="s">
@@ -12178,7 +12152,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45744</v>
       </c>
       <c r="F199" t="s">
@@ -12219,7 +12193,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>45744</v>
       </c>
       <c r="F200" t="s">
@@ -12260,7 +12234,7 @@
       <c r="C201">
         <v>2026</v>
       </c>
-      <c r="D201" s="2">
+      <c r="D201" s="1">
         <v>46408</v>
       </c>
       <c r="F201" t="s">
@@ -12304,7 +12278,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>45898</v>
       </c>
       <c r="F202" t="s">
@@ -12345,7 +12319,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>45971</v>
       </c>
       <c r="F203" t="s">
@@ -12386,7 +12360,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>45744</v>
       </c>
       <c r="F204" t="s">
@@ -12427,7 +12401,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>46092</v>
       </c>
       <c r="F205" t="s">
@@ -12468,7 +12442,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46204</v>
       </c>
       <c r="F206" t="s">
@@ -12512,7 +12486,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46185</v>
       </c>
       <c r="H207" t="s">
@@ -12547,7 +12521,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45890</v>
       </c>
       <c r="G208" t="s">
@@ -12585,7 +12559,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>46185</v>
       </c>
       <c r="H209" t="s">
@@ -12620,7 +12594,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>46175</v>
       </c>
       <c r="F210" t="s">
@@ -12661,7 +12635,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45890</v>
       </c>
       <c r="G211" t="s">
@@ -12699,7 +12673,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46175</v>
       </c>
       <c r="F212" t="s">
@@ -12740,7 +12714,7 @@
       <c r="C213">
         <v>2026</v>
       </c>
-      <c r="D213" s="2">
+      <c r="D213" s="1">
         <v>46185</v>
       </c>
       <c r="G213" t="s">
@@ -12778,7 +12752,7 @@
       <c r="C214">
         <v>2026</v>
       </c>
-      <c r="D214" s="2">
+      <c r="D214" s="1">
         <v>45890</v>
       </c>
       <c r="G214" t="s">
@@ -12816,7 +12790,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45890</v>
       </c>
       <c r="G215" t="s">
@@ -12854,7 +12828,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>45890</v>
       </c>
       <c r="G216" t="s">
@@ -12892,7 +12866,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>46175</v>
       </c>
       <c r="F217" t="s">
@@ -12933,7 +12907,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45890</v>
       </c>
       <c r="G218" t="s">
@@ -12971,7 +12945,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>46119</v>
       </c>
       <c r="F219" t="s">
@@ -13012,7 +12986,7 @@
       <c r="C220">
         <v>2026</v>
       </c>
-      <c r="D220" s="2">
+      <c r="D220" s="1">
         <v>46119</v>
       </c>
       <c r="F220" t="s">
@@ -13053,7 +13027,7 @@
       <c r="C221">
         <v>2026</v>
       </c>
-      <c r="D221" s="2">
+      <c r="D221" s="1">
         <v>46119</v>
       </c>
       <c r="F221" t="s">
@@ -13094,7 +13068,7 @@
       <c r="C222">
         <v>2026</v>
       </c>
-      <c r="D222" s="2">
+      <c r="D222" s="1">
         <v>45856</v>
       </c>
       <c r="F222" t="s">
@@ -13135,7 +13109,7 @@
       <c r="C223">
         <v>2026</v>
       </c>
-      <c r="D223" s="2">
+      <c r="D223" s="1">
         <v>45769</v>
       </c>
       <c r="F223" t="s">
@@ -13176,7 +13150,7 @@
       <c r="C224">
         <v>2026</v>
       </c>
-      <c r="D224" s="2">
+      <c r="D224" s="1">
         <v>45769</v>
       </c>
       <c r="F224" t="s">
@@ -13217,7 +13191,7 @@
       <c r="C225">
         <v>2026</v>
       </c>
-      <c r="D225" s="2">
+      <c r="D225" s="1">
         <v>45769</v>
       </c>
       <c r="F225" t="s">
@@ -13258,7 +13232,7 @@
       <c r="C226">
         <v>2026</v>
       </c>
-      <c r="D226" s="2">
+      <c r="D226" s="1">
         <v>45769</v>
       </c>
       <c r="F226" t="s">
@@ -13299,7 +13273,7 @@
       <c r="C227">
         <v>2026</v>
       </c>
-      <c r="D227" s="2">
+      <c r="D227" s="1">
         <v>45769</v>
       </c>
       <c r="F227" t="s">
@@ -13340,7 +13314,7 @@
       <c r="C228">
         <v>2026</v>
       </c>
-      <c r="D228" s="2">
+      <c r="D228" s="1">
         <v>45769</v>
       </c>
       <c r="F228" t="s">
@@ -13381,7 +13355,7 @@
       <c r="C229">
         <v>2026</v>
       </c>
-      <c r="D229" s="2">
+      <c r="D229" s="1">
         <v>45769</v>
       </c>
       <c r="F229" t="s">
@@ -13422,7 +13396,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>46147</v>
       </c>
       <c r="H230" t="s">
@@ -13457,7 +13431,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>46147</v>
       </c>
       <c r="H231" t="s">
@@ -13492,7 +13466,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>46147</v>
       </c>
       <c r="H232" t="s">
@@ -13527,7 +13501,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45814</v>
       </c>
       <c r="F233" t="s">
@@ -13568,7 +13542,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45860</v>
       </c>
       <c r="F234" t="s">
@@ -13609,7 +13583,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -13650,7 +13624,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45863</v>
       </c>
       <c r="F236" t="s">
@@ -13691,7 +13665,7 @@
       <c r="C237">
         <v>2026</v>
       </c>
-      <c r="D237" s="2">
+      <c r="D237" s="1">
         <v>45905</v>
       </c>
       <c r="G237" t="s">
@@ -13729,7 +13703,7 @@
       <c r="C238">
         <v>2026</v>
       </c>
-      <c r="D238" s="2">
+      <c r="D238" s="1">
         <v>45971</v>
       </c>
       <c r="F238" t="s">
@@ -13770,7 +13744,7 @@
       <c r="C239">
         <v>2026</v>
       </c>
-      <c r="D239" s="2">
+      <c r="D239" s="1">
         <v>45971</v>
       </c>
       <c r="F239" t="s">
@@ -13811,7 +13785,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45744</v>
       </c>
       <c r="F240" t="s">
@@ -13852,7 +13826,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45814</v>
       </c>
       <c r="F241" t="s">
@@ -13893,7 +13867,7 @@
       <c r="C242">
         <v>2026</v>
       </c>
-      <c r="D242" s="2">
+      <c r="D242" s="1">
         <v>45807</v>
       </c>
       <c r="F242" t="s">
@@ -13934,7 +13908,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45802</v>
       </c>
       <c r="F243" t="s">
@@ -13975,7 +13949,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45802</v>
       </c>
       <c r="F244" t="s">
@@ -14016,7 +13990,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45802</v>
       </c>
       <c r="F245" t="s">
@@ -14057,7 +14031,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45897</v>
       </c>
       <c r="H246" t="s">
@@ -14092,7 +14066,7 @@
       <c r="C247">
         <v>2026</v>
       </c>
-      <c r="D247" s="2">
+      <c r="D247" s="1">
         <v>45802</v>
       </c>
       <c r="F247" t="s">
@@ -14133,7 +14107,7 @@
       <c r="C248">
         <v>2026</v>
       </c>
-      <c r="D248" s="2">
+      <c r="D248" s="1">
         <v>45802</v>
       </c>
       <c r="F248" t="s">
@@ -14174,7 +14148,7 @@
       <c r="C249">
         <v>2026</v>
       </c>
-      <c r="D249" s="2">
+      <c r="D249" s="1">
         <v>45876</v>
       </c>
       <c r="F249" t="s">
@@ -14215,7 +14189,7 @@
       <c r="C250">
         <v>2026</v>
       </c>
-      <c r="D250" s="2">
+      <c r="D250" s="1">
         <v>45889</v>
       </c>
       <c r="F250" t="s">
@@ -14256,7 +14230,7 @@
       <c r="C251">
         <v>2026</v>
       </c>
-      <c r="D251" s="2">
+      <c r="D251" s="1">
         <v>45876</v>
       </c>
       <c r="F251" t="s">
@@ -14297,7 +14271,7 @@
       <c r="C252">
         <v>2026</v>
       </c>
-      <c r="D252" s="2">
+      <c r="D252" s="1">
         <v>45926</v>
       </c>
       <c r="F252" t="s">
@@ -14338,7 +14312,7 @@
       <c r="C253">
         <v>2026</v>
       </c>
-      <c r="D253" s="2">
+      <c r="D253" s="1">
         <v>45909</v>
       </c>
       <c r="F253" t="s">
@@ -14379,7 +14353,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -14420,7 +14394,7 @@
       <c r="C255">
         <v>2026</v>
       </c>
-      <c r="D255" s="2">
+      <c r="D255" s="1">
         <v>46119</v>
       </c>
       <c r="F255" t="s">
@@ -14461,7 +14435,7 @@
       <c r="C256">
         <v>2026</v>
       </c>
-      <c r="D256" s="2">
+      <c r="D256" s="1">
         <v>46119</v>
       </c>
       <c r="F256" t="s">
@@ -14502,7 +14476,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>46086</v>
       </c>
       <c r="G257" t="s">
@@ -14540,7 +14514,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45965</v>
       </c>
       <c r="F258" t="s">
@@ -14581,7 +14555,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46064</v>
       </c>
       <c r="H259" t="s">
@@ -14613,7 +14587,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>46049</v>
       </c>
       <c r="F260" t="s">
@@ -14654,7 +14628,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45996</v>
       </c>
       <c r="G261" t="s">
@@ -14692,7 +14666,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45996</v>
       </c>
       <c r="G262" t="s">
@@ -14730,7 +14704,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45989</v>
       </c>
       <c r="G263" t="s">
@@ -14768,7 +14742,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46156</v>
       </c>
       <c r="H264" t="s">
@@ -14803,7 +14777,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45996</v>
       </c>
       <c r="G265" t="s">
@@ -14841,7 +14815,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45989</v>
       </c>
       <c r="G266" t="s">
@@ -14879,7 +14853,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>46002</v>
       </c>
       <c r="G267" t="s">
@@ -14917,7 +14891,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46002</v>
       </c>
       <c r="G268" t="s">
@@ -14955,7 +14929,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>45996</v>
       </c>
       <c r="G269" t="s">
@@ -14993,7 +14967,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46002</v>
       </c>
       <c r="G270" t="s">
@@ -15031,7 +15005,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>46031</v>
       </c>
       <c r="G271" t="s">
@@ -15069,7 +15043,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46153</v>
       </c>
       <c r="F272" t="s">
@@ -15110,7 +15084,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46135</v>
       </c>
       <c r="F273" t="s">
@@ -15151,7 +15125,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>46230</v>
       </c>
       <c r="F274" t="s">
@@ -15192,7 +15166,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>45996</v>
       </c>
       <c r="G275" t="s">
@@ -15230,7 +15204,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>45996</v>
       </c>
       <c r="G276" t="s">
@@ -15268,7 +15242,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>46164</v>
       </c>
       <c r="H277" t="s">
@@ -15303,7 +15277,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>46020</v>
       </c>
       <c r="G278" t="s">
@@ -15341,7 +15315,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>46225</v>
       </c>
       <c r="F279" t="s">
@@ -15385,7 +15359,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46176</v>
       </c>
       <c r="H280" t="s">
@@ -15420,7 +15394,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>46086</v>
       </c>
       <c r="G281" t="s">
@@ -15458,7 +15432,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46052</v>
       </c>
       <c r="G282" t="s">
@@ -15534,7 +15508,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46010</v>
       </c>
       <c r="G284" t="s">
@@ -15572,7 +15546,7 @@
       <c r="C285">
         <v>2026</v>
       </c>
-      <c r="D285" s="2">
+      <c r="D285" s="1">
         <v>46010</v>
       </c>
       <c r="G285" t="s">
@@ -15610,7 +15584,7 @@
       <c r="C286">
         <v>2026</v>
       </c>
-      <c r="D286" s="2">
+      <c r="D286" s="1">
         <v>46079</v>
       </c>
       <c r="F286" t="s">
@@ -15651,7 +15625,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>46010</v>
       </c>
       <c r="G287" t="s">
@@ -15689,7 +15663,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>46010</v>
       </c>
       <c r="G288" t="s">
@@ -15727,7 +15701,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>46230</v>
       </c>
       <c r="F289" t="s">
@@ -15771,7 +15745,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>46063</v>
       </c>
       <c r="G290" t="s">
@@ -15809,7 +15783,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>46063</v>
       </c>
       <c r="F291" t="s">
@@ -15850,7 +15824,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>46063</v>
       </c>
       <c r="F292" t="s">
@@ -15891,7 +15865,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>46063</v>
       </c>
       <c r="F293" t="s">
@@ -15932,7 +15906,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>46063</v>
       </c>
       <c r="G294" t="s">
@@ -15970,7 +15944,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46114</v>
       </c>
       <c r="F295" t="s">
@@ -16011,7 +15985,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46191</v>
       </c>
       <c r="F296" t="s">
@@ -16052,7 +16026,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46230</v>
       </c>
       <c r="F297" t="s">
@@ -16093,7 +16067,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>46230</v>
       </c>
       <c r="F298" t="s">
@@ -16134,7 +16108,7 @@
       <c r="C299">
         <v>2026</v>
       </c>
-      <c r="D299" s="2">
+      <c r="D299" s="1">
         <v>46230</v>
       </c>
       <c r="F299" t="s">
@@ -16175,7 +16149,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>46230</v>
       </c>
       <c r="F300" t="s">
@@ -16216,7 +16190,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>46230</v>
       </c>
       <c r="F301" t="s">
@@ -16257,7 +16231,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>46230</v>
       </c>
       <c r="F302" t="s">
@@ -16298,7 +16272,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>46230</v>
       </c>
       <c r="F303" t="s">
@@ -16339,7 +16313,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45996</v>
       </c>
       <c r="G304" t="s">
@@ -16377,7 +16351,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>46052</v>
       </c>
       <c r="F305" t="s">
@@ -16418,7 +16392,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>46057</v>
       </c>
       <c r="F306" t="s">
@@ -16459,7 +16433,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>46112</v>
       </c>
       <c r="F307" t="s">
@@ -16500,7 +16474,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>46063</v>
       </c>
       <c r="G308" t="s">
@@ -16538,7 +16512,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>46048</v>
       </c>
       <c r="G309" t="s">
@@ -16576,7 +16550,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>46063</v>
       </c>
       <c r="H310" t="s">
@@ -16611,7 +16585,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>46119</v>
       </c>
       <c r="F311" t="s">
@@ -16652,7 +16626,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>46119</v>
       </c>
       <c r="F312" t="s">
@@ -16693,7 +16667,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>46113</v>
       </c>
       <c r="F313" t="s">
@@ -16734,7 +16708,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>46104</v>
       </c>
       <c r="F314" t="s">
@@ -16775,7 +16749,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>46135</v>
       </c>
       <c r="H315" t="s">
@@ -16810,7 +16784,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>46230</v>
       </c>
       <c r="F316" t="s">
@@ -16851,7 +16825,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>46086</v>
       </c>
       <c r="G317" t="s">
@@ -16889,7 +16863,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>46086</v>
       </c>
       <c r="G318" t="s">
@@ -16927,7 +16901,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>46086</v>
       </c>
       <c r="H319" t="s">
@@ -16962,7 +16936,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46230</v>
       </c>
       <c r="F320" t="s">
@@ -17003,7 +16977,7 @@
       <c r="C321">
         <v>2026</v>
       </c>
-      <c r="D321" s="2">
+      <c r="D321" s="1">
         <v>46176</v>
       </c>
       <c r="H321" t="s">
@@ -17038,7 +17012,7 @@
       <c r="C322">
         <v>2026</v>
       </c>
-      <c r="D322" s="2">
+      <c r="D322" s="1">
         <v>46147</v>
       </c>
       <c r="H322" t="s">
@@ -17073,7 +17047,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46135</v>
       </c>
       <c r="H323" t="s">
@@ -17108,7 +17082,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46227</v>
       </c>
       <c r="G324" t="s">
@@ -17149,7 +17123,7 @@
       <c r="C325">
         <v>2026</v>
       </c>
-      <c r="D325" s="2">
+      <c r="D325" s="1">
         <v>46230</v>
       </c>
       <c r="F325" t="s">
@@ -17190,7 +17164,7 @@
       <c r="C326">
         <v>2026</v>
       </c>
-      <c r="D326" s="2">
+      <c r="D326" s="1">
         <v>46083</v>
       </c>
       <c r="F326" t="s">
@@ -17231,7 +17205,7 @@
       <c r="C327">
         <v>2026</v>
       </c>
-      <c r="D327" s="2">
+      <c r="D327" s="1">
         <v>46083</v>
       </c>
       <c r="G327" t="s">
@@ -17269,7 +17243,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46083</v>
       </c>
       <c r="F328" t="s">
@@ -17310,7 +17284,7 @@
       <c r="C329">
         <v>2026</v>
       </c>
-      <c r="D329" s="2">
+      <c r="D329" s="1">
         <v>46127</v>
       </c>
       <c r="F329" t="s">
@@ -17351,7 +17325,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>46100</v>
       </c>
       <c r="F330" t="s">
@@ -17392,7 +17366,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46230</v>
       </c>
       <c r="F331" t="s">
@@ -17433,7 +17407,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46079</v>
       </c>
       <c r="H332" t="s">
@@ -17468,7 +17442,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>46176</v>
       </c>
       <c r="F333" t="s">
@@ -17509,7 +17483,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>46176</v>
       </c>
       <c r="F334" t="s">
@@ -17550,7 +17524,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>46155</v>
       </c>
       <c r="F335" t="s">
@@ -17591,7 +17565,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46155</v>
       </c>
       <c r="G336" t="s">
@@ -17629,7 +17603,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>46129</v>
       </c>
       <c r="F337" t="s">
@@ -17670,7 +17644,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>46119</v>
       </c>
       <c r="F338" t="s">
@@ -17711,7 +17685,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46135</v>
       </c>
       <c r="H339" t="s">
@@ -17746,7 +17720,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46127</v>
       </c>
       <c r="H340" t="s">
@@ -17781,7 +17755,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>46127</v>
       </c>
       <c r="H341" t="s">
@@ -17816,7 +17790,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46175</v>
       </c>
       <c r="F342" t="s">
@@ -17857,7 +17831,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46139</v>
       </c>
       <c r="H343" t="s">
@@ -17892,7 +17866,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46155</v>
       </c>
       <c r="H344" t="s">
@@ -17927,7 +17901,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46175</v>
       </c>
       <c r="F345" t="s">
@@ -17968,7 +17942,7 @@
       <c r="C346">
         <v>2026</v>
       </c>
-      <c r="D346" s="2">
+      <c r="D346" s="1">
         <v>46156</v>
       </c>
       <c r="F346" t="s">
@@ -18009,7 +17983,7 @@
       <c r="C347">
         <v>2026</v>
       </c>
-      <c r="D347" s="2">
+      <c r="D347" s="1">
         <v>46157</v>
       </c>
       <c r="G347" t="s">
@@ -18047,7 +18021,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46183</v>
       </c>
       <c r="H348" t="s">
@@ -18082,7 +18056,7 @@
       <c r="C349">
         <v>2026</v>
       </c>
-      <c r="D349" s="2">
+      <c r="D349" s="1">
         <v>46183</v>
       </c>
       <c r="H349" t="s">
@@ -18117,7 +18091,7 @@
       <c r="C350">
         <v>2026</v>
       </c>
-      <c r="D350" s="2">
+      <c r="D350" s="1">
         <v>46230</v>
       </c>
       <c r="F350" t="s">
@@ -18161,7 +18135,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>46185</v>
       </c>
       <c r="H351" t="s">
@@ -18196,7 +18170,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>46185</v>
       </c>
       <c r="H352" t="s">
@@ -18231,7 +18205,7 @@
       <c r="C353">
         <v>2026</v>
       </c>
-      <c r="D353" s="2">
+      <c r="D353" s="1">
         <v>46175</v>
       </c>
       <c r="F353" t="s">
@@ -18272,7 +18246,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46175</v>
       </c>
       <c r="F354" t="s">
@@ -18313,7 +18287,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46230</v>
       </c>
       <c r="F355" t="s">
@@ -18354,7 +18328,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46175</v>
       </c>
       <c r="G356" t="s">
@@ -18392,7 +18366,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46175</v>
       </c>
       <c r="G357" t="s">
@@ -18430,7 +18404,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46175</v>
       </c>
       <c r="G358" t="s">
@@ -18468,7 +18442,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46230</v>
       </c>
       <c r="F359" t="s">
@@ -18509,7 +18483,7 @@
       <c r="C360">
         <v>2026</v>
       </c>
-      <c r="D360" s="2">
+      <c r="D360" s="1">
         <v>46175</v>
       </c>
       <c r="G360" t="s">
@@ -18547,7 +18521,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46175</v>
       </c>
       <c r="G361" t="s">
@@ -18585,7 +18559,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46175</v>
       </c>
       <c r="G362" t="s">
@@ -18623,7 +18597,7 @@
       <c r="C363">
         <v>2026</v>
       </c>
-      <c r="D363" s="2">
+      <c r="D363" s="1">
         <v>46230</v>
       </c>
       <c r="F363" t="s">
@@ -18664,7 +18638,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46209</v>
       </c>
       <c r="F364" t="s">
@@ -18708,7 +18682,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46230</v>
       </c>
       <c r="F365" t="s">
@@ -18749,7 +18723,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46230</v>
       </c>
       <c r="F366" t="s">
@@ -18790,7 +18764,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -18831,7 +18805,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46230</v>
       </c>
       <c r="F368" t="s">
@@ -18872,7 +18846,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46230</v>
       </c>
       <c r="F369" t="s">
@@ -18913,7 +18887,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46230</v>
       </c>
       <c r="F370" t="s">
@@ -18957,7 +18931,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46230</v>
       </c>
       <c r="F371" t="s">
@@ -18998,7 +18972,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46157</v>
       </c>
       <c r="G372" t="s">
@@ -19036,7 +19010,7 @@
       <c r="C373">
         <v>2026</v>
       </c>
-      <c r="D373" s="2">
+      <c r="D373" s="1">
         <v>46213</v>
       </c>
       <c r="F373" t="s">
@@ -19080,7 +19054,7 @@
       <c r="C374">
         <v>2026</v>
       </c>
-      <c r="D374" s="2">
+      <c r="D374" s="1">
         <v>46205</v>
       </c>
       <c r="F374" t="s">
@@ -19124,7 +19098,7 @@
       <c r="C375">
         <v>2026</v>
       </c>
-      <c r="D375" s="2">
+      <c r="D375" s="1">
         <v>46176</v>
       </c>
       <c r="F375" t="s">
@@ -19165,7 +19139,7 @@
       <c r="C376">
         <v>2026</v>
       </c>
-      <c r="D376" s="2">
+      <c r="D376" s="1">
         <v>46150</v>
       </c>
       <c r="F376" t="s">
@@ -19206,7 +19180,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46220</v>
       </c>
       <c r="F377" t="s">
@@ -19250,7 +19224,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46224</v>
       </c>
       <c r="F378" t="s">
@@ -19294,7 +19268,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46155</v>
       </c>
       <c r="H379" t="s">
@@ -19329,7 +19303,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46156</v>
       </c>
       <c r="F380" t="s">
@@ -19370,7 +19344,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46185</v>
       </c>
       <c r="H381" t="s">
@@ -19405,7 +19379,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -19446,7 +19420,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -19487,7 +19461,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -19528,7 +19502,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -19569,7 +19543,7 @@
       <c r="C386">
         <v>2026</v>
       </c>
-      <c r="D386" s="2">
+      <c r="D386" s="1">
         <v>46230</v>
       </c>
       <c r="F386" t="s">
@@ -19610,7 +19584,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>46147</v>
       </c>
       <c r="G387" t="s">
@@ -19648,7 +19622,7 @@
       <c r="C388">
         <v>2026</v>
       </c>
-      <c r="D388" s="2">
+      <c r="D388" s="1">
         <v>46164</v>
       </c>
       <c r="F388" t="s">
@@ -19689,7 +19663,7 @@
       <c r="C389">
         <v>2026</v>
       </c>
-      <c r="D389" s="2">
+      <c r="D389" s="1">
         <v>46230</v>
       </c>
       <c r="F389" t="s">
@@ -19730,7 +19704,7 @@
       <c r="C390">
         <v>2026</v>
       </c>
-      <c r="D390" s="2">
+      <c r="D390" s="1">
         <v>46171</v>
       </c>
       <c r="F390" t="s">
@@ -19771,7 +19745,7 @@
       <c r="C391">
         <v>2026</v>
       </c>
-      <c r="D391" s="2">
+      <c r="D391" s="1">
         <v>46176</v>
       </c>
       <c r="G391" t="s">
@@ -19809,7 +19783,7 @@
       <c r="C392">
         <v>2026</v>
       </c>
-      <c r="D392" s="2">
+      <c r="D392" s="1">
         <v>46230</v>
       </c>
       <c r="F392" t="s">
@@ -19850,7 +19824,7 @@
       <c r="C393">
         <v>2026</v>
       </c>
-      <c r="D393" s="2">
+      <c r="D393" s="1">
         <v>46211</v>
       </c>
       <c r="F393" t="s">
@@ -19894,7 +19868,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46183</v>
       </c>
       <c r="H394" t="s">
@@ -19929,7 +19903,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46191</v>
       </c>
       <c r="H395" t="s">
@@ -19964,7 +19938,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46191</v>
       </c>
       <c r="G396" t="s">
@@ -20002,7 +19976,7 @@
       <c r="C397">
         <v>2026</v>
       </c>
-      <c r="D397" s="2">
+      <c r="D397" s="1">
         <v>46230</v>
       </c>
       <c r="F397" t="s">
@@ -20043,7 +20017,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46230</v>
       </c>
       <c r="F398" t="s">
@@ -20084,7 +20058,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46191</v>
       </c>
       <c r="G399" t="s">
@@ -20122,7 +20096,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46191</v>
       </c>
       <c r="G400" t="s">
@@ -20160,7 +20134,7 @@
       <c r="C401">
         <v>2026</v>
       </c>
-      <c r="D401" s="2">
+      <c r="D401" s="1">
         <v>46230</v>
       </c>
       <c r="F401" t="s">
@@ -20204,7 +20178,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46226</v>
       </c>
       <c r="F402" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (25/08/2026 08:32)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5153,8 +5153,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5170,7 +5178,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5178,12 +5186,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5483,52 +5509,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5606,7 +5632,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5743,7 +5769,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5880,7 +5906,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5921,7 +5947,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5956,7 +5982,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -5997,7 +6023,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6035,7 +6061,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6076,7 +6102,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6117,7 +6143,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6155,7 +6181,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6196,7 +6222,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6237,7 +6263,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6278,7 +6304,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6319,7 +6345,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6421,7 +6447,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6462,7 +6488,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6503,7 +6529,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6544,7 +6570,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6585,7 +6611,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6626,7 +6652,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6699,7 +6725,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6772,7 +6798,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6813,7 +6839,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6854,7 +6880,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6895,7 +6921,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6968,7 +6994,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7073,7 +7099,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="2">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7114,7 +7140,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7155,7 +7181,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7196,7 +7222,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7237,7 +7263,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="2">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7278,7 +7304,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="2">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7316,7 +7342,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="2">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7357,7 +7383,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="2">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7398,7 +7424,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="2">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7471,7 +7497,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="2">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7512,7 +7538,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="2">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7585,7 +7611,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="2">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7658,7 +7684,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="2">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7731,7 +7757,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="2">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7801,7 +7827,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="2">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7874,7 +7900,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="2">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7909,7 +7935,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="2">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7950,7 +7976,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="2">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -7991,7 +8017,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="2">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8032,7 +8058,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="2">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8073,7 +8099,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="2">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8114,7 +8140,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="2">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8155,7 +8181,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="2">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8196,7 +8222,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="2">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8231,7 +8257,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="2">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8272,7 +8298,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="2">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8310,7 +8336,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="2">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8348,7 +8374,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="2">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8386,7 +8412,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="2">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8424,7 +8450,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="2">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8465,7 +8491,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="2">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8506,7 +8532,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="2">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8547,7 +8573,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="2">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8588,7 +8614,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="2">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8629,7 +8655,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="2">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8670,7 +8696,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="2">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8711,7 +8737,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="2">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8752,7 +8778,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="2">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8831,7 +8857,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="2">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8872,7 +8898,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="2">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8913,7 +8939,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="2">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8954,7 +8980,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="2">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -8995,7 +9021,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="2">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9036,7 +9062,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="2">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9077,7 +9103,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="2">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9118,7 +9144,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="2">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9191,7 +9217,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="2">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9232,7 +9258,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="2">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9273,7 +9299,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="2">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9314,7 +9340,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="2">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9355,7 +9381,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="2">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9393,7 +9419,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="2">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9463,7 +9489,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="2">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9504,7 +9530,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="2">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9545,7 +9571,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="2">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9586,7 +9612,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="2">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9688,7 +9714,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="2">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9729,7 +9755,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="2">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9770,7 +9796,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="2">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9811,7 +9837,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="2">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9849,7 +9875,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="2">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9887,7 +9913,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="2">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9928,7 +9954,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="2">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9969,7 +9995,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="2">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10010,7 +10036,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="2">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10051,7 +10077,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="2">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10092,7 +10118,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="2">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10133,7 +10159,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="2">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10174,7 +10200,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="2">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10215,7 +10241,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="2">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10253,7 +10279,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="2">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10294,7 +10320,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="2">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10335,7 +10361,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="2">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10405,7 +10431,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="2">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10478,7 +10504,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="2">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10519,7 +10545,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="2">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10560,7 +10586,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="2">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10633,7 +10659,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="2">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10674,7 +10700,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="2">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10715,7 +10741,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="2">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10753,7 +10779,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="2">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10826,7 +10852,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="2">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10864,7 +10890,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="2">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10934,7 +10960,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="2">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11039,7 +11065,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="2">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11080,7 +11106,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="2">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11121,7 +11147,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="2">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11162,7 +11188,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="2">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11203,7 +11229,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="2">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11244,7 +11270,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="2">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11285,7 +11311,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="2">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11358,7 +11384,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="2">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11399,7 +11425,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="2">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11440,7 +11466,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="2">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11481,7 +11507,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="2">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11551,7 +11577,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="2">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11592,7 +11618,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="2">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11633,7 +11659,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="2">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11674,7 +11700,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="2">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11715,7 +11741,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="2">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11756,7 +11782,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="2">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11794,7 +11820,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="2">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11867,7 +11893,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="2">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11908,7 +11934,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="2">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11946,7 +11972,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="2">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -11981,7 +12007,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="2">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12022,7 +12048,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="2">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12063,7 +12089,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="2">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12142,7 +12168,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173" s="2">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12183,7 +12209,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174" s="2">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12224,7 +12250,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175" s="2">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12265,7 +12291,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176" s="2">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12306,7 +12332,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177" s="2">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12347,7 +12373,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178" s="2">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12388,7 +12414,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179" s="2">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12429,7 +12455,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180" s="2">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12502,7 +12528,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182" s="2">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12569,7 +12595,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="1">
+      <c r="D184" s="2">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12642,7 +12668,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="1">
+      <c r="D186" s="2">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12683,7 +12709,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D187" s="2">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12724,7 +12750,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="1">
+      <c r="D188" s="2">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12765,7 +12791,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="1">
+      <c r="D189" s="2">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12806,7 +12832,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="1">
+      <c r="D190" s="2">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12847,7 +12873,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="1">
+      <c r="D191" s="2">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12920,7 +12946,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="1">
+      <c r="D193" s="2">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12961,7 +12987,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="1">
+      <c r="D194" s="2">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13002,7 +13028,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="1">
+      <c r="D195" s="2">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13043,7 +13069,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="2">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13084,7 +13110,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="1">
+      <c r="D197" s="2">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13125,7 +13151,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="1">
+      <c r="D198" s="2">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13163,7 +13189,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="1">
+      <c r="D199" s="2">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13204,7 +13230,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="1">
+      <c r="D200" s="2">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13283,7 +13309,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="1">
+      <c r="D202" s="2">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13324,7 +13350,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="1">
+      <c r="D203" s="2">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13365,7 +13391,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="1">
+      <c r="D204" s="2">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13406,7 +13432,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="1">
+      <c r="D205" s="2">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13444,7 +13470,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="1">
+      <c r="D206" s="2">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13485,7 +13511,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="1">
+      <c r="D207" s="2">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13526,7 +13552,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="1">
+      <c r="D208" s="2">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13564,7 +13590,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="1">
+      <c r="D209" s="2">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13605,7 +13631,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="1">
+      <c r="D210" s="2">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13646,7 +13672,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="1">
+      <c r="D211" s="2">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13687,7 +13713,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="1">
+      <c r="D212" s="2">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13801,7 +13827,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="1">
+      <c r="D215" s="2">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13842,7 +13868,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="1">
+      <c r="D216" s="2">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13883,7 +13909,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="1">
+      <c r="D217" s="2">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13924,7 +13950,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="1">
+      <c r="D218" s="2">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13965,7 +13991,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="1">
+      <c r="D219" s="2">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14326,7 +14352,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="1">
+      <c r="D230" s="2">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14367,7 +14393,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="1">
+      <c r="D231" s="2">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14408,7 +14434,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="1">
+      <c r="D232" s="2">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14449,7 +14475,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="1">
+      <c r="D233" s="2">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14490,7 +14516,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="1">
+      <c r="D234" s="2">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14531,7 +14557,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="1">
+      <c r="D235" s="2">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14572,7 +14598,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="1">
+      <c r="D236" s="2">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14709,7 +14735,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="1">
+      <c r="D240" s="2">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14750,7 +14776,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="1">
+      <c r="D241" s="2">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14823,7 +14849,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="1">
+      <c r="D243" s="2">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14864,7 +14890,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="1">
+      <c r="D244" s="2">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14902,7 +14928,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="1">
+      <c r="D245" s="2">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14940,7 +14966,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="1">
+      <c r="D246" s="2">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15202,7 +15228,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="1">
+      <c r="D254" s="2">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15307,7 +15333,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="1">
+      <c r="D257" s="2">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15348,7 +15374,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="1">
+      <c r="D258" s="2">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15389,7 +15415,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="1">
+      <c r="D259" s="2">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15430,7 +15456,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="1">
+      <c r="D260" s="2">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15468,7 +15494,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="1">
+      <c r="D261" s="2">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15509,7 +15535,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="1">
+      <c r="D262" s="2">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15550,7 +15576,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D263" s="2">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15591,7 +15617,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D264" s="2">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15635,7 +15661,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D265" s="2">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15676,7 +15702,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="1">
+      <c r="D266" s="2">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15717,7 +15743,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="1">
+      <c r="D267" s="2">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15758,7 +15784,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="1">
+      <c r="D268" s="2">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15799,7 +15825,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="1">
+      <c r="D269" s="2">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15843,7 +15869,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="1">
+      <c r="D270" s="2">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15878,7 +15904,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="1">
+      <c r="D271" s="2">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15916,7 +15942,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="1">
+      <c r="D272" s="2">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15951,7 +15977,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="1">
+      <c r="D273" s="2">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -15992,7 +16018,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="1">
+      <c r="D274" s="2">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16030,7 +16056,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="1">
+      <c r="D275" s="2">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16071,7 +16097,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="1">
+      <c r="D276" s="2">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16109,7 +16135,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="1">
+      <c r="D277" s="2">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16147,7 +16173,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="1">
+      <c r="D278" s="2">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16185,7 +16211,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="1">
+      <c r="D279" s="2">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16223,7 +16249,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="1">
+      <c r="D280" s="2">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16264,7 +16290,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="1">
+      <c r="D281" s="2">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16302,7 +16328,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="1">
+      <c r="D282" s="2">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16343,7 +16369,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="1">
+      <c r="D283" s="2">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16384,7 +16410,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="1">
+      <c r="D284" s="2">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16489,7 +16515,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="1">
+      <c r="D287" s="2">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16530,7 +16556,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="1">
+      <c r="D288" s="2">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16571,7 +16597,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="1">
+      <c r="D289" s="2">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16612,7 +16638,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="1">
+      <c r="D290" s="2">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16653,7 +16679,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="1">
+      <c r="D291" s="2">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16694,7 +16720,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="1">
+      <c r="D292" s="2">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16735,7 +16761,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="1">
+      <c r="D293" s="2">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16776,7 +16802,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="1">
+      <c r="D294" s="2">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16817,7 +16843,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="1">
+      <c r="D295" s="2">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16852,7 +16878,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="1">
+      <c r="D296" s="2">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16887,7 +16913,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="1">
+      <c r="D297" s="2">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16922,7 +16948,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="1">
+      <c r="D298" s="2">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -16995,7 +17021,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="1">
+      <c r="D300" s="2">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17036,7 +17062,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="1">
+      <c r="D301" s="2">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17077,7 +17103,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="1">
+      <c r="D302" s="2">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17118,7 +17144,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="1">
+      <c r="D303" s="2">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17156,7 +17182,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="1">
+      <c r="D304" s="2">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17197,7 +17223,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="1">
+      <c r="D305" s="2">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17238,7 +17264,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="1">
+      <c r="D306" s="2">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17279,7 +17305,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="1">
+      <c r="D307" s="2">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17320,7 +17346,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="1">
+      <c r="D308" s="2">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17361,7 +17387,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="1">
+      <c r="D309" s="2">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17402,7 +17428,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="1">
+      <c r="D310" s="2">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17443,7 +17469,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="1">
+      <c r="D311" s="2">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17484,7 +17510,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="1">
+      <c r="D312" s="2">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17519,7 +17545,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="1">
+      <c r="D313" s="2">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17560,7 +17586,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="1">
+      <c r="D314" s="2">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17601,7 +17627,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="1">
+      <c r="D315" s="2">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17642,7 +17668,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="1">
+      <c r="D316" s="2">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17683,7 +17709,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="1">
+      <c r="D317" s="2">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17724,7 +17750,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="1">
+      <c r="D318" s="2">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17765,7 +17791,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="1">
+      <c r="D319" s="2">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17806,7 +17832,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="1">
+      <c r="D320" s="2">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17911,7 +17937,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="1">
+      <c r="D323" s="2">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17952,7 +17978,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="1">
+      <c r="D324" s="2">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18089,7 +18115,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="1">
+      <c r="D328" s="2">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18159,7 +18185,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="1">
+      <c r="D330" s="2">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18200,7 +18226,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="1">
+      <c r="D331" s="2">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18232,7 +18258,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="1">
+      <c r="D332" s="2">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18273,7 +18299,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="1">
+      <c r="D333" s="2">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18311,7 +18337,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="1">
+      <c r="D334" s="2">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18349,7 +18375,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="1">
+      <c r="D335" s="2">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18387,7 +18413,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="1">
+      <c r="D336" s="2">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18422,7 +18448,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="1">
+      <c r="D337" s="2">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18460,7 +18486,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="1">
+      <c r="D338" s="2">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18498,7 +18524,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="1">
+      <c r="D339" s="2">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18536,7 +18562,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="1">
+      <c r="D340" s="2">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18574,7 +18600,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="1">
+      <c r="D341" s="2">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18612,7 +18638,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="1">
+      <c r="D342" s="2">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18650,7 +18676,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="1">
+      <c r="D343" s="2">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18688,7 +18714,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="1">
+      <c r="D344" s="2">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18729,7 +18755,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="1">
+      <c r="D345" s="2">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18834,7 +18860,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="1">
+      <c r="D348" s="2">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18939,7 +18965,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="1">
+      <c r="D351" s="2">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -18977,7 +19003,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="1">
+      <c r="D352" s="2">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19047,7 +19073,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="1">
+      <c r="D354" s="2">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19082,7 +19108,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="1">
+      <c r="D355" s="2">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19120,7 +19146,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="1">
+      <c r="D356" s="2">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19164,7 +19190,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="1">
+      <c r="D357" s="2">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19199,7 +19225,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="1">
+      <c r="D358" s="2">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19237,7 +19263,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="1">
+      <c r="D359" s="2">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19313,7 +19339,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="1">
+      <c r="D361" s="2">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19351,7 +19377,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="1">
+      <c r="D362" s="2">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19421,7 +19447,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="1">
+      <c r="D364" s="2">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19462,7 +19488,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="1">
+      <c r="D365" s="2">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19500,7 +19526,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="1">
+      <c r="D366" s="2">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19538,7 +19564,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="1">
+      <c r="D367" s="2">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19582,7 +19608,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="1">
+      <c r="D368" s="2">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19620,7 +19646,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="1">
+      <c r="D369" s="2">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19661,7 +19687,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="1">
+      <c r="D370" s="2">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19702,7 +19728,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="1">
+      <c r="D371" s="2">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19743,7 +19769,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="1">
+      <c r="D372" s="2">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19909,7 +19935,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="1">
+      <c r="D377" s="2">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19950,7 +19976,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="1">
+      <c r="D378" s="2">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -19991,7 +20017,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="1">
+      <c r="D379" s="2">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20032,7 +20058,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="1">
+      <c r="D380" s="2">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20073,7 +20099,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="1">
+      <c r="D381" s="2">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20114,7 +20140,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="1">
+      <c r="D382" s="2">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20155,7 +20181,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="1">
+      <c r="D383" s="2">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20196,7 +20222,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="1">
+      <c r="D384" s="2">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20237,7 +20263,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="1">
+      <c r="D385" s="2">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20310,7 +20336,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="1">
+      <c r="D387" s="2">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20540,7 +20566,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="1">
+      <c r="D394" s="2">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20581,7 +20607,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="1">
+      <c r="D395" s="2">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20622,7 +20648,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="1">
+      <c r="D396" s="2">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20695,7 +20721,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="1">
+      <c r="D398" s="2">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20733,7 +20759,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="1">
+      <c r="D399" s="2">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20771,7 +20797,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="1">
+      <c r="D400" s="2">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20838,7 +20864,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="1">
+      <c r="D402" s="2">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20911,7 +20937,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="1">
+      <c r="D404" s="2">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20952,7 +20978,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="1">
+      <c r="D405" s="2">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -20993,7 +21019,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="1">
+      <c r="D406" s="2">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21034,7 +21060,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="1">
+      <c r="D407" s="2">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21101,7 +21127,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="1">
+      <c r="D409" s="2">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21142,7 +21168,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="1">
+      <c r="D410" s="2">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21180,7 +21206,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="1">
+      <c r="D411" s="2">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21218,7 +21244,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="1">
+      <c r="D412" s="2">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21253,7 +21279,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="1">
+      <c r="D413" s="2">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21390,7 +21416,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="1">
+      <c r="D417" s="2">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21425,7 +21451,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="1">
+      <c r="D418" s="2">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21460,7 +21486,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="1">
+      <c r="D419" s="2">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21527,7 +21553,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="1">
+      <c r="D421" s="2">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21568,7 +21594,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="1">
+      <c r="D422" s="2">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21609,7 +21635,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="1">
+      <c r="D423" s="2">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21650,7 +21676,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="1">
+      <c r="D424" s="2">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21688,7 +21714,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="1">
+      <c r="D425" s="2">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21729,7 +21755,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="1">
+      <c r="D426" s="2">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21770,7 +21796,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="1">
+      <c r="D427" s="2">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21968,7 +21994,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="1">
+      <c r="D433" s="2">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22009,7 +22035,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="1">
+      <c r="D434" s="2">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22140,7 +22166,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="1">
+      <c r="D438" s="2">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22181,7 +22207,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="1">
+      <c r="D439" s="2">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22222,7 +22248,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="1">
+      <c r="D440" s="2">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22263,7 +22289,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="1">
+      <c r="D441" s="2">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22301,7 +22327,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="1">
+      <c r="D442" s="2">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22342,7 +22368,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="1">
+      <c r="D443" s="2">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22383,7 +22409,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="1">
+      <c r="D444" s="2">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22418,7 +22444,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="1">
+      <c r="D445" s="2">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22453,7 +22479,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="1">
+      <c r="D446" s="2">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22520,7 +22546,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="1">
+      <c r="D448" s="2">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22561,7 +22587,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="1">
+      <c r="D449" s="2">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22596,7 +22622,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="1">
+      <c r="D450" s="2">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22631,7 +22657,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="1">
+      <c r="D451" s="2">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22704,7 +22730,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="1">
+      <c r="D453" s="2">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22745,7 +22771,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="1">
+      <c r="D454" s="2">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22783,7 +22809,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="1">
+      <c r="D455" s="2">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22818,7 +22844,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="1">
+      <c r="D456" s="2">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22917,7 +22943,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="1">
+      <c r="D459" s="2">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22961,7 +22987,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="1">
+      <c r="D460" s="2">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23028,7 +23054,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="1">
+      <c r="D462" s="2">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23127,7 +23153,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="1">
+      <c r="D465" s="2">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23168,7 +23194,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="1">
+      <c r="D466" s="2">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23209,7 +23235,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="1">
+      <c r="D467" s="2">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23250,7 +23276,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="1">
+      <c r="D468" s="2">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23288,7 +23314,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="1">
+      <c r="D469" s="2">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23326,7 +23352,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="1">
+      <c r="D470" s="2">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23364,7 +23390,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="1">
+      <c r="D471" s="2">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23405,7 +23431,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="1">
+      <c r="D472" s="2">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23443,7 +23469,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="1">
+      <c r="D473" s="2">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23481,7 +23507,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="1">
+      <c r="D474" s="2">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23519,7 +23545,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="1">
+      <c r="D475" s="2">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23592,7 +23618,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="1">
+      <c r="D477" s="2">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23764,7 +23790,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="1">
+      <c r="D482" s="2">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23805,7 +23831,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="1">
+      <c r="D483" s="2">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23846,7 +23872,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="1">
+      <c r="D484" s="2">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24111,7 +24137,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="1">
+      <c r="D492" s="2">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24152,7 +24178,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="1">
+      <c r="D493" s="2">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24257,7 +24283,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="1">
+      <c r="D496" s="2">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24301,7 +24327,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="1">
+      <c r="D497" s="2">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24342,7 +24368,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="1">
+      <c r="D498" s="2">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24380,7 +24406,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="1">
+      <c r="D499" s="2">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24456,7 +24482,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="1">
+      <c r="D501" s="2">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24500,7 +24526,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="1">
+      <c r="D502" s="2">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24541,7 +24567,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="1">
+      <c r="D503" s="2">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24646,7 +24672,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="1">
+      <c r="D506" s="2">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24690,7 +24716,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="1">
+      <c r="D507" s="2">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24766,7 +24792,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="1">
+      <c r="D509" s="2">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24801,7 +24827,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="1">
+      <c r="D510" s="2">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24842,7 +24868,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="1">
+      <c r="D511" s="2">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24877,7 +24903,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="1">
+      <c r="D512" s="2">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24918,7 +24944,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="1">
+      <c r="D513" s="2">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24959,7 +24985,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="1">
+      <c r="D514" s="2">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25000,7 +25026,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="1">
+      <c r="D515" s="2">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25041,7 +25067,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="1">
+      <c r="D516" s="2">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25146,7 +25172,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="1">
+      <c r="D519" s="2">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25280,7 +25306,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="1">
+      <c r="D523" s="2">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25417,7 +25443,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="1">
+      <c r="D527" s="2">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25554,7 +25580,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="1">
+      <c r="D531" s="2">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25659,7 +25685,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="1">
+      <c r="D534" s="2">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25697,7 +25723,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="1">
+      <c r="D535" s="2">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25898,7 +25924,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="1">
+      <c r="D541" s="2">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25942,7 +25968,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="1">
+      <c r="D542" s="2">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -25977,7 +26003,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="1">
+      <c r="D543" s="2">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26012,7 +26038,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="1">
+      <c r="D544" s="2">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26210,7 +26236,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="1">
+      <c r="D550" s="2">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26315,7 +26341,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="1">
+      <c r="D553" s="2">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26356,7 +26382,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="1">
+      <c r="D554" s="2">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26522,7 +26548,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="1">
+      <c r="D559" s="2">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26720,7 +26746,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="1">
+      <c r="D565" s="2">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27340,7 +27366,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="1">
+      <c r="D584" s="2">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (25/08/2026 08:37)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5153,16 +5153,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5178,7 +5170,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5186,30 +5178,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5509,52 +5483,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5632,7 +5606,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5769,7 +5743,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5906,7 +5880,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5947,7 +5921,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5982,7 +5956,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6023,7 +5997,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6061,7 +6035,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6102,7 +6076,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6143,7 +6117,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6181,7 +6155,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6222,7 +6196,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6263,7 +6237,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6304,7 +6278,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6345,7 +6319,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6447,7 +6421,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6488,7 +6462,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6529,7 +6503,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6570,7 +6544,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6611,7 +6585,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6652,7 +6626,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6725,7 +6699,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6798,7 +6772,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6839,7 +6813,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6880,7 +6854,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6921,7 +6895,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6994,7 +6968,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7099,7 +7073,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7140,7 +7114,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7181,7 +7155,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7222,7 +7196,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7263,7 +7237,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7304,7 +7278,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7342,7 +7316,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7383,7 +7357,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7424,7 +7398,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7497,7 +7471,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7538,7 +7512,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7611,7 +7585,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7684,7 +7658,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7757,7 +7731,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7827,7 +7801,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7900,7 +7874,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7935,7 +7909,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7976,7 +7950,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8017,7 +7991,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8058,7 +8032,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8099,7 +8073,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8140,7 +8114,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8181,7 +8155,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8222,7 +8196,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8257,7 +8231,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8298,7 +8272,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8336,7 +8310,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8374,7 +8348,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8412,7 +8386,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8450,7 +8424,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8491,7 +8465,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8532,7 +8506,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8573,7 +8547,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8614,7 +8588,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8655,7 +8629,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8696,7 +8670,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8737,7 +8711,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8778,7 +8752,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8857,7 +8831,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8898,7 +8872,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8939,7 +8913,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8980,7 +8954,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9021,7 +8995,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9062,7 +9036,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9103,7 +9077,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9144,7 +9118,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9217,7 +9191,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9258,7 +9232,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9299,7 +9273,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9340,7 +9314,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9381,7 +9355,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9419,7 +9393,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9489,7 +9463,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9530,7 +9504,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9571,7 +9545,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9612,7 +9586,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9714,7 +9688,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9755,7 +9729,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9796,7 +9770,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9837,7 +9811,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9875,7 +9849,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9913,7 +9887,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9954,7 +9928,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9995,7 +9969,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10036,7 +10010,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10077,7 +10051,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10118,7 +10092,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10159,7 +10133,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10200,7 +10174,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10241,7 +10215,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10279,7 +10253,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10320,7 +10294,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10361,7 +10335,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10431,7 +10405,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10504,7 +10478,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10545,7 +10519,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10586,7 +10560,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10659,7 +10633,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10700,7 +10674,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10741,7 +10715,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10779,7 +10753,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10852,7 +10826,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10890,7 +10864,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10960,7 +10934,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11065,7 +11039,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11106,7 +11080,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11147,7 +11121,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11188,7 +11162,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11229,7 +11203,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11270,7 +11244,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11311,7 +11285,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11384,7 +11358,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11425,7 +11399,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11466,7 +11440,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11507,7 +11481,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11577,7 +11551,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11618,7 +11592,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11659,7 +11633,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11700,7 +11674,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11741,7 +11715,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11782,7 +11756,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11820,7 +11794,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11893,7 +11867,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11934,7 +11908,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11972,7 +11946,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12007,7 +11981,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12048,7 +12022,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12089,7 +12063,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12168,7 +12142,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12209,7 +12183,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12250,7 +12224,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12291,7 +12265,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12332,7 +12306,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12373,7 +12347,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12414,7 +12388,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12455,7 +12429,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12528,7 +12502,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12595,7 +12569,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12668,7 +12642,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12709,7 +12683,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12750,7 +12724,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12791,7 +12765,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12832,7 +12806,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12873,7 +12847,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12946,7 +12920,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12987,7 +12961,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13028,7 +13002,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13069,7 +13043,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13110,7 +13084,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13151,7 +13125,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13189,7 +13163,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13230,7 +13204,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13309,7 +13283,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13350,7 +13324,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13391,7 +13365,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13432,7 +13406,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13470,7 +13444,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13511,7 +13485,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13552,7 +13526,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13590,7 +13564,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13631,7 +13605,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13672,7 +13646,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13713,7 +13687,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13827,7 +13801,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13868,7 +13842,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13909,7 +13883,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13950,7 +13924,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13991,7 +13965,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14352,7 +14326,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14393,7 +14367,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14434,7 +14408,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14475,7 +14449,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14516,7 +14490,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14557,7 +14531,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14598,7 +14572,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14735,7 +14709,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14776,7 +14750,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14849,7 +14823,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14890,7 +14864,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14928,7 +14902,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14966,7 +14940,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15228,7 +15202,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15333,7 +15307,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15374,7 +15348,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15415,7 +15389,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15456,7 +15430,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15494,7 +15468,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15535,7 +15509,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15576,7 +15550,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15617,7 +15591,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15661,7 +15635,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15702,7 +15676,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15743,7 +15717,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15784,7 +15758,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15825,7 +15799,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15869,7 +15843,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15904,7 +15878,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15942,7 +15916,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15977,7 +15951,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16018,7 +15992,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16056,7 +16030,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16097,7 +16071,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16135,7 +16109,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16173,7 +16147,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16211,7 +16185,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16249,7 +16223,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16290,7 +16264,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16328,7 +16302,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16369,7 +16343,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16410,7 +16384,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16515,7 +16489,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16556,7 +16530,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16597,7 +16571,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16638,7 +16612,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16679,7 +16653,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16720,7 +16694,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16761,7 +16735,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16802,7 +16776,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16843,7 +16817,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16878,7 +16852,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16913,7 +16887,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16948,7 +16922,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17021,7 +16995,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17062,7 +17036,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17103,7 +17077,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17144,7 +17118,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17182,7 +17156,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17223,7 +17197,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17264,7 +17238,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17305,7 +17279,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17346,7 +17320,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17387,7 +17361,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17428,7 +17402,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17469,7 +17443,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17510,7 +17484,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17545,7 +17519,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17586,7 +17560,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17627,7 +17601,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17668,7 +17642,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17709,7 +17683,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17750,7 +17724,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17791,7 +17765,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17832,7 +17806,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17937,7 +17911,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17978,7 +17952,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18115,7 +18089,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18185,7 +18159,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18226,7 +18200,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18258,7 +18232,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18299,7 +18273,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18337,7 +18311,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18375,7 +18349,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18413,7 +18387,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18448,7 +18422,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18486,7 +18460,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18524,7 +18498,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18562,7 +18536,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18600,7 +18574,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18638,7 +18612,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18676,7 +18650,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18714,7 +18688,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18755,7 +18729,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18860,7 +18834,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18965,7 +18939,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19003,7 +18977,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19073,7 +19047,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19108,7 +19082,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19146,7 +19120,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19190,7 +19164,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19225,7 +19199,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19263,7 +19237,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19339,7 +19313,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19377,7 +19351,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19447,7 +19421,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19488,7 +19462,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19526,7 +19500,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19564,7 +19538,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19608,7 +19582,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19646,7 +19620,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19687,7 +19661,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19728,7 +19702,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19769,7 +19743,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19935,7 +19909,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19976,7 +19950,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20017,7 +19991,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20058,7 +20032,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20099,7 +20073,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20140,7 +20114,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20181,7 +20155,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20222,7 +20196,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20263,7 +20237,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20336,7 +20310,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20566,7 +20540,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20607,7 +20581,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20648,7 +20622,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20721,7 +20695,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20759,7 +20733,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20797,7 +20771,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20864,7 +20838,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20937,7 +20911,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20978,7 +20952,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21019,7 +20993,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21060,7 +21034,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21127,7 +21101,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21168,7 +21142,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21206,7 +21180,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21244,7 +21218,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21279,7 +21253,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21416,7 +21390,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21451,7 +21425,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21486,7 +21460,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21553,7 +21527,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21594,7 +21568,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21635,7 +21609,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21676,7 +21650,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21714,7 +21688,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21755,7 +21729,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21796,7 +21770,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21994,7 +21968,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22035,7 +22009,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22166,7 +22140,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22207,7 +22181,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22248,7 +22222,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22289,7 +22263,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22327,7 +22301,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22368,7 +22342,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22409,7 +22383,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22444,7 +22418,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22479,7 +22453,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22546,7 +22520,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22587,7 +22561,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22622,7 +22596,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22657,7 +22631,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22730,7 +22704,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22771,7 +22745,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22809,7 +22783,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22844,7 +22818,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22943,7 +22917,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22987,7 +22961,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23054,7 +23028,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23153,7 +23127,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23194,7 +23168,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23235,7 +23209,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23276,7 +23250,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23314,7 +23288,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23352,7 +23326,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23390,7 +23364,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23431,7 +23405,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23469,7 +23443,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23507,7 +23481,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23545,7 +23519,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23618,7 +23592,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23790,7 +23764,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23831,7 +23805,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23872,7 +23846,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24137,7 +24111,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24178,7 +24152,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24283,7 +24257,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24327,7 +24301,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24368,7 +24342,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24406,7 +24380,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24482,7 +24456,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24526,7 +24500,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24567,7 +24541,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24672,7 +24646,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24716,7 +24690,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24792,7 +24766,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24827,7 +24801,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24868,7 +24842,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24903,7 +24877,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24944,7 +24918,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24985,7 +24959,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25026,7 +25000,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25067,7 +25041,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25172,7 +25146,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25306,7 +25280,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25443,7 +25417,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25580,7 +25554,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25685,7 +25659,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25723,7 +25697,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25924,7 +25898,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25968,7 +25942,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26003,7 +25977,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26038,7 +26012,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26236,7 +26210,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26341,7 +26315,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26382,7 +26356,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26548,7 +26522,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26746,7 +26720,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27366,7 +27340,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (10/09/2026 09:01)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,8 +5159,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5176,7 +5184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5184,12 +5192,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5489,52 +5515,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5749,7 +5775,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5886,7 +5912,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5927,7 +5953,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5962,7 +5988,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6003,7 +6029,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6041,7 +6067,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6082,7 +6108,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6123,7 +6149,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6161,7 +6187,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6202,7 +6228,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6243,7 +6269,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6284,7 +6310,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6325,7 +6351,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6427,7 +6453,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6468,7 +6494,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6509,7 +6535,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6550,7 +6576,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6591,7 +6617,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6632,7 +6658,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6705,7 +6731,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6778,7 +6804,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6819,7 +6845,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6860,7 +6886,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6901,7 +6927,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6974,7 +7000,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7079,7 +7105,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="2">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7120,7 +7146,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7161,7 +7187,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7202,7 +7228,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7243,7 +7269,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="2">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7284,7 +7310,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="2">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7322,7 +7348,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="2">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7363,7 +7389,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="2">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7404,7 +7430,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="2">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7477,7 +7503,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="2">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7518,7 +7544,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="2">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7591,7 +7617,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="2">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7664,7 +7690,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="2">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7737,7 +7763,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="2">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7807,7 +7833,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="2">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7880,7 +7906,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="2">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7915,7 +7941,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="2">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7956,7 +7982,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="2">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -7997,7 +8023,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="2">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8038,7 +8064,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="2">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8079,7 +8105,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="2">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8120,7 +8146,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="2">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8161,7 +8187,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="2">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8202,7 +8228,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="2">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8237,7 +8263,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="2">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8278,7 +8304,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="2">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8316,7 +8342,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="2">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8354,7 +8380,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="2">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8392,7 +8418,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="2">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8430,7 +8456,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="2">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8471,7 +8497,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="2">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8512,7 +8538,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="2">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8553,7 +8579,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="2">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8594,7 +8620,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="2">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8635,7 +8661,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="2">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8676,7 +8702,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="2">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8717,7 +8743,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="2">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8758,7 +8784,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="2">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8837,7 +8863,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="2">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8878,7 +8904,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="2">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8919,7 +8945,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="2">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8960,7 +8986,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="2">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9001,7 +9027,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="2">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9042,7 +9068,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="2">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9083,7 +9109,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="2">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9124,7 +9150,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="2">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9197,7 +9223,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="2">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9238,7 +9264,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="2">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9279,7 +9305,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="2">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9320,7 +9346,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="2">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9361,7 +9387,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="2">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9399,7 +9425,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="2">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9469,7 +9495,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="2">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9510,7 +9536,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="2">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9551,7 +9577,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="2">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9592,7 +9618,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="2">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9694,7 +9720,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="2">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9735,7 +9761,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="2">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9776,7 +9802,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="2">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9817,7 +9843,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="2">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9855,7 +9881,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="2">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9893,7 +9919,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="2">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9934,7 +9960,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="2">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9975,7 +10001,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="2">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10016,7 +10042,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="2">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10057,7 +10083,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="2">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10098,7 +10124,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="2">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10139,7 +10165,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="2">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10180,7 +10206,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="2">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10221,7 +10247,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="2">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10259,7 +10285,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="2">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10300,7 +10326,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="2">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10341,7 +10367,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="2">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10411,7 +10437,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="2">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10484,7 +10510,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="2">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10525,7 +10551,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="2">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10566,7 +10592,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="2">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10639,7 +10665,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="2">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10680,7 +10706,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="2">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10721,7 +10747,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="2">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10759,7 +10785,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="2">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10832,7 +10858,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="2">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10870,7 +10896,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="2">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10940,7 +10966,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="2">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11045,7 +11071,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="2">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11086,7 +11112,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="2">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11127,7 +11153,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="2">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11168,7 +11194,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="2">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11209,7 +11235,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="2">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11250,7 +11276,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="2">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11291,7 +11317,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="2">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11364,7 +11390,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="2">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11405,7 +11431,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="2">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11446,7 +11472,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="2">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11487,7 +11513,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="2">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11557,7 +11583,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="2">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11598,7 +11624,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="2">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11639,7 +11665,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="2">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11680,7 +11706,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="2">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11721,7 +11747,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="2">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11762,7 +11788,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="2">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11800,7 +11826,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="2">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11873,7 +11899,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="2">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11914,7 +11940,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="2">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11952,7 +11978,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="2">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -11987,7 +12013,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="2">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12028,7 +12054,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="2">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12069,7 +12095,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="2">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12148,7 +12174,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173" s="2">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12189,7 +12215,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174" s="2">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12230,7 +12256,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175" s="2">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12271,7 +12297,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176" s="2">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12312,7 +12338,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177" s="2">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12353,7 +12379,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178" s="2">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12394,7 +12420,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179" s="2">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12435,7 +12461,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180" s="2">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12508,7 +12534,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182" s="2">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12575,7 +12601,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="1">
+      <c r="D184" s="2">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12648,7 +12674,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="1">
+      <c r="D186" s="2">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12689,7 +12715,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D187" s="2">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12730,7 +12756,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="1">
+      <c r="D188" s="2">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12771,7 +12797,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="1">
+      <c r="D189" s="2">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12812,7 +12838,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="1">
+      <c r="D190" s="2">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12853,7 +12879,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="1">
+      <c r="D191" s="2">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12926,7 +12952,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="1">
+      <c r="D193" s="2">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12967,7 +12993,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="1">
+      <c r="D194" s="2">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13008,7 +13034,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="1">
+      <c r="D195" s="2">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13049,7 +13075,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="2">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13090,7 +13116,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="1">
+      <c r="D197" s="2">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13131,7 +13157,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="1">
+      <c r="D198" s="2">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13169,7 +13195,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="1">
+      <c r="D199" s="2">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13210,7 +13236,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="1">
+      <c r="D200" s="2">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13289,7 +13315,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="1">
+      <c r="D202" s="2">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13330,7 +13356,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="1">
+      <c r="D203" s="2">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13371,7 +13397,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="1">
+      <c r="D204" s="2">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13412,7 +13438,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="1">
+      <c r="D205" s="2">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13450,7 +13476,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="1">
+      <c r="D206" s="2">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13491,7 +13517,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="1">
+      <c r="D207" s="2">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13532,7 +13558,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="1">
+      <c r="D208" s="2">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13570,7 +13596,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="1">
+      <c r="D209" s="2">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13611,7 +13637,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="1">
+      <c r="D210" s="2">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13652,7 +13678,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="1">
+      <c r="D211" s="2">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13693,7 +13719,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="1">
+      <c r="D212" s="2">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13807,7 +13833,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="1">
+      <c r="D215" s="2">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13848,7 +13874,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="1">
+      <c r="D216" s="2">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13889,7 +13915,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="1">
+      <c r="D217" s="2">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13930,7 +13956,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="1">
+      <c r="D218" s="2">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13971,7 +13997,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="1">
+      <c r="D219" s="2">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14332,7 +14358,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="1">
+      <c r="D230" s="2">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14373,7 +14399,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="1">
+      <c r="D231" s="2">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14414,7 +14440,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="1">
+      <c r="D232" s="2">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14455,7 +14481,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="1">
+      <c r="D233" s="2">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14496,7 +14522,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="1">
+      <c r="D234" s="2">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14537,7 +14563,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="1">
+      <c r="D235" s="2">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14578,7 +14604,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="1">
+      <c r="D236" s="2">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14715,7 +14741,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="1">
+      <c r="D240" s="2">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14756,7 +14782,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="1">
+      <c r="D241" s="2">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14829,7 +14855,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="1">
+      <c r="D243" s="2">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14870,7 +14896,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="1">
+      <c r="D244" s="2">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14908,7 +14934,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="1">
+      <c r="D245" s="2">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14946,7 +14972,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="1">
+      <c r="D246" s="2">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15208,7 +15234,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="1">
+      <c r="D254" s="2">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15313,7 +15339,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="1">
+      <c r="D257" s="2">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15354,7 +15380,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="1">
+      <c r="D258" s="2">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15395,7 +15421,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="1">
+      <c r="D259" s="2">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15436,7 +15462,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="1">
+      <c r="D260" s="2">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15474,7 +15500,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="1">
+      <c r="D261" s="2">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15515,7 +15541,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="1">
+      <c r="D262" s="2">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15556,7 +15582,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D263" s="2">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15597,7 +15623,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D264" s="2">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15641,7 +15667,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D265" s="2">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15682,7 +15708,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="1">
+      <c r="D266" s="2">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15723,7 +15749,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="1">
+      <c r="D267" s="2">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15764,7 +15790,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="1">
+      <c r="D268" s="2">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15805,7 +15831,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="1">
+      <c r="D269" s="2">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15849,7 +15875,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="1">
+      <c r="D270" s="2">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15884,7 +15910,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="1">
+      <c r="D271" s="2">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15922,7 +15948,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="1">
+      <c r="D272" s="2">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15957,7 +15983,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="1">
+      <c r="D273" s="2">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -15998,7 +16024,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="1">
+      <c r="D274" s="2">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16036,7 +16062,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="1">
+      <c r="D275" s="2">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16077,7 +16103,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="1">
+      <c r="D276" s="2">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16115,7 +16141,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="1">
+      <c r="D277" s="2">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16153,7 +16179,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="1">
+      <c r="D278" s="2">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16191,7 +16217,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="1">
+      <c r="D279" s="2">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16229,7 +16255,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="1">
+      <c r="D280" s="2">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16270,7 +16296,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="1">
+      <c r="D281" s="2">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16308,7 +16334,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="1">
+      <c r="D282" s="2">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16349,7 +16375,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="1">
+      <c r="D283" s="2">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16390,7 +16416,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="1">
+      <c r="D284" s="2">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16495,7 +16521,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="1">
+      <c r="D287" s="2">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16536,7 +16562,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="1">
+      <c r="D288" s="2">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16577,7 +16603,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="1">
+      <c r="D289" s="2">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16618,7 +16644,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="1">
+      <c r="D290" s="2">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16659,7 +16685,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="1">
+      <c r="D291" s="2">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16700,7 +16726,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="1">
+      <c r="D292" s="2">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16741,7 +16767,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="1">
+      <c r="D293" s="2">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16782,7 +16808,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="1">
+      <c r="D294" s="2">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16823,7 +16849,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="1">
+      <c r="D295" s="2">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16858,7 +16884,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="1">
+      <c r="D296" s="2">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16893,7 +16919,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="1">
+      <c r="D297" s="2">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16928,7 +16954,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="1">
+      <c r="D298" s="2">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17001,7 +17027,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="1">
+      <c r="D300" s="2">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17042,7 +17068,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="1">
+      <c r="D301" s="2">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17083,7 +17109,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="1">
+      <c r="D302" s="2">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17124,7 +17150,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="1">
+      <c r="D303" s="2">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17162,7 +17188,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="1">
+      <c r="D304" s="2">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17203,7 +17229,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="1">
+      <c r="D305" s="2">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17244,7 +17270,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="1">
+      <c r="D306" s="2">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17285,7 +17311,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="1">
+      <c r="D307" s="2">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17326,7 +17352,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="1">
+      <c r="D308" s="2">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17367,7 +17393,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="1">
+      <c r="D309" s="2">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17408,7 +17434,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="1">
+      <c r="D310" s="2">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17449,7 +17475,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="1">
+      <c r="D311" s="2">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17490,7 +17516,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="1">
+      <c r="D312" s="2">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17525,7 +17551,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="1">
+      <c r="D313" s="2">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17566,7 +17592,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="1">
+      <c r="D314" s="2">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17607,7 +17633,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="1">
+      <c r="D315" s="2">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17648,7 +17674,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="1">
+      <c r="D316" s="2">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17689,7 +17715,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="1">
+      <c r="D317" s="2">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17730,7 +17756,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="1">
+      <c r="D318" s="2">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17771,7 +17797,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="1">
+      <c r="D319" s="2">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17812,7 +17838,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="1">
+      <c r="D320" s="2">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17917,7 +17943,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="1">
+      <c r="D323" s="2">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17958,7 +17984,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="1">
+      <c r="D324" s="2">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18095,7 +18121,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="1">
+      <c r="D328" s="2">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18165,7 +18191,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="1">
+      <c r="D330" s="2">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18206,7 +18232,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="1">
+      <c r="D331" s="2">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18238,7 +18264,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="1">
+      <c r="D332" s="2">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18279,7 +18305,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="1">
+      <c r="D333" s="2">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18317,7 +18343,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="1">
+      <c r="D334" s="2">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18355,7 +18381,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="1">
+      <c r="D335" s="2">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18393,7 +18419,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="1">
+      <c r="D336" s="2">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18428,7 +18454,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="1">
+      <c r="D337" s="2">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18466,7 +18492,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="1">
+      <c r="D338" s="2">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18504,7 +18530,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="1">
+      <c r="D339" s="2">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18542,7 +18568,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="1">
+      <c r="D340" s="2">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18580,7 +18606,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="1">
+      <c r="D341" s="2">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18618,7 +18644,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="1">
+      <c r="D342" s="2">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18656,7 +18682,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="1">
+      <c r="D343" s="2">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18694,7 +18720,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="1">
+      <c r="D344" s="2">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18735,7 +18761,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="1">
+      <c r="D345" s="2">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18840,7 +18866,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="1">
+      <c r="D348" s="2">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18945,7 +18971,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="1">
+      <c r="D351" s="2">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -18983,7 +19009,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="1">
+      <c r="D352" s="2">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19053,7 +19079,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="1">
+      <c r="D354" s="2">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19088,7 +19114,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="1">
+      <c r="D355" s="2">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19126,7 +19152,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="1">
+      <c r="D356" s="2">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19170,7 +19196,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="1">
+      <c r="D357" s="2">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19205,7 +19231,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="1">
+      <c r="D358" s="2">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19243,7 +19269,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="1">
+      <c r="D359" s="2">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19319,7 +19345,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="1">
+      <c r="D361" s="2">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19357,7 +19383,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="1">
+      <c r="D362" s="2">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19427,7 +19453,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="1">
+      <c r="D364" s="2">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19468,7 +19494,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="1">
+      <c r="D365" s="2">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19506,7 +19532,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="1">
+      <c r="D366" s="2">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19544,7 +19570,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="1">
+      <c r="D367" s="2">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19588,7 +19614,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="1">
+      <c r="D368" s="2">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19626,7 +19652,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="1">
+      <c r="D369" s="2">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19667,7 +19693,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="1">
+      <c r="D370" s="2">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19708,7 +19734,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="1">
+      <c r="D371" s="2">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19749,7 +19775,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="1">
+      <c r="D372" s="2">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19915,7 +19941,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="1">
+      <c r="D377" s="2">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19956,7 +19982,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="1">
+      <c r="D378" s="2">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -19997,7 +20023,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="1">
+      <c r="D379" s="2">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20038,7 +20064,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="1">
+      <c r="D380" s="2">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20079,7 +20105,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="1">
+      <c r="D381" s="2">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20120,7 +20146,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="1">
+      <c r="D382" s="2">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20161,7 +20187,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="1">
+      <c r="D383" s="2">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20202,7 +20228,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="1">
+      <c r="D384" s="2">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20243,7 +20269,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="1">
+      <c r="D385" s="2">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20316,7 +20342,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="1">
+      <c r="D387" s="2">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20546,7 +20572,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="1">
+      <c r="D394" s="2">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20587,7 +20613,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="1">
+      <c r="D395" s="2">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20628,7 +20654,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="1">
+      <c r="D396" s="2">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20701,7 +20727,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="1">
+      <c r="D398" s="2">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20739,7 +20765,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="1">
+      <c r="D399" s="2">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20777,7 +20803,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="1">
+      <c r="D400" s="2">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20844,7 +20870,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="1">
+      <c r="D402" s="2">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20917,7 +20943,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="1">
+      <c r="D404" s="2">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20958,7 +20984,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="1">
+      <c r="D405" s="2">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -20999,7 +21025,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="1">
+      <c r="D406" s="2">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21040,7 +21066,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="1">
+      <c r="D407" s="2">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21107,7 +21133,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="1">
+      <c r="D409" s="2">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21148,7 +21174,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="1">
+      <c r="D410" s="2">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21186,7 +21212,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="1">
+      <c r="D411" s="2">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21224,7 +21250,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="1">
+      <c r="D412" s="2">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21259,7 +21285,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="1">
+      <c r="D413" s="2">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21396,7 +21422,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="1">
+      <c r="D417" s="2">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21431,7 +21457,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="1">
+      <c r="D418" s="2">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21466,7 +21492,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="1">
+      <c r="D419" s="2">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21533,7 +21559,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="1">
+      <c r="D421" s="2">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21574,7 +21600,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="1">
+      <c r="D422" s="2">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21615,7 +21641,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="1">
+      <c r="D423" s="2">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21656,7 +21682,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="1">
+      <c r="D424" s="2">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21694,7 +21720,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="1">
+      <c r="D425" s="2">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21735,7 +21761,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="1">
+      <c r="D426" s="2">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21776,7 +21802,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="1">
+      <c r="D427" s="2">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21974,7 +22000,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="1">
+      <c r="D433" s="2">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22015,7 +22041,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="1">
+      <c r="D434" s="2">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22146,7 +22172,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="1">
+      <c r="D438" s="2">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22187,7 +22213,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="1">
+      <c r="D439" s="2">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22228,7 +22254,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="1">
+      <c r="D440" s="2">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22269,7 +22295,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="1">
+      <c r="D441" s="2">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22307,7 +22333,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="1">
+      <c r="D442" s="2">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22348,7 +22374,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="1">
+      <c r="D443" s="2">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22389,7 +22415,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="1">
+      <c r="D444" s="2">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22424,7 +22450,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="1">
+      <c r="D445" s="2">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22459,7 +22485,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="1">
+      <c r="D446" s="2">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22526,7 +22552,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="1">
+      <c r="D448" s="2">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22567,7 +22593,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="1">
+      <c r="D449" s="2">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22602,7 +22628,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="1">
+      <c r="D450" s="2">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22637,7 +22663,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="1">
+      <c r="D451" s="2">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22710,7 +22736,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="1">
+      <c r="D453" s="2">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22751,7 +22777,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="1">
+      <c r="D454" s="2">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22789,7 +22815,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="1">
+      <c r="D455" s="2">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22824,7 +22850,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="1">
+      <c r="D456" s="2">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22923,7 +22949,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="1">
+      <c r="D459" s="2">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22967,7 +22993,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="1">
+      <c r="D460" s="2">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23034,7 +23060,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="1">
+      <c r="D462" s="2">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23133,7 +23159,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="1">
+      <c r="D465" s="2">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23174,7 +23200,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="1">
+      <c r="D466" s="2">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23215,7 +23241,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="1">
+      <c r="D467" s="2">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23256,7 +23282,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="1">
+      <c r="D468" s="2">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23294,7 +23320,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="1">
+      <c r="D469" s="2">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23332,7 +23358,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="1">
+      <c r="D470" s="2">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23370,7 +23396,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="1">
+      <c r="D471" s="2">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23411,7 +23437,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="1">
+      <c r="D472" s="2">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23449,7 +23475,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="1">
+      <c r="D473" s="2">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23487,7 +23513,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="1">
+      <c r="D474" s="2">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23525,7 +23551,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="1">
+      <c r="D475" s="2">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23598,7 +23624,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="1">
+      <c r="D477" s="2">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23770,7 +23796,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="1">
+      <c r="D482" s="2">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23811,7 +23837,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="1">
+      <c r="D483" s="2">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23852,7 +23878,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="1">
+      <c r="D484" s="2">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24117,7 +24143,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="1">
+      <c r="D492" s="2">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24158,7 +24184,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="1">
+      <c r="D493" s="2">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24263,7 +24289,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="1">
+      <c r="D496" s="2">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24307,7 +24333,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="1">
+      <c r="D497" s="2">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24348,7 +24374,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="1">
+      <c r="D498" s="2">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24386,7 +24412,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="1">
+      <c r="D499" s="2">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24462,7 +24488,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="1">
+      <c r="D501" s="2">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24506,7 +24532,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="1">
+      <c r="D502" s="2">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24547,7 +24573,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="1">
+      <c r="D503" s="2">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24652,7 +24678,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="1">
+      <c r="D506" s="2">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24696,7 +24722,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="1">
+      <c r="D507" s="2">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24772,7 +24798,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="1">
+      <c r="D509" s="2">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24807,7 +24833,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="1">
+      <c r="D510" s="2">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24848,7 +24874,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="1">
+      <c r="D511" s="2">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24883,7 +24909,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="1">
+      <c r="D512" s="2">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24924,7 +24950,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="1">
+      <c r="D513" s="2">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24965,7 +24991,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="1">
+      <c r="D514" s="2">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25006,7 +25032,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="1">
+      <c r="D515" s="2">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25047,7 +25073,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="1">
+      <c r="D516" s="2">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25152,7 +25178,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="1">
+      <c r="D519" s="2">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25286,7 +25312,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="1">
+      <c r="D523" s="2">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25423,7 +25449,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="1">
+      <c r="D527" s="2">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25560,7 +25586,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="1">
+      <c r="D531" s="2">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25665,7 +25691,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="1">
+      <c r="D534" s="2">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25703,7 +25729,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="1">
+      <c r="D535" s="2">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25904,7 +25930,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="1">
+      <c r="D541" s="2">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25948,7 +25974,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="1">
+      <c r="D542" s="2">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -25983,7 +26009,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="1">
+      <c r="D543" s="2">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26018,7 +26044,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="1">
+      <c r="D544" s="2">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26216,7 +26242,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="1">
+      <c r="D550" s="2">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26321,7 +26347,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="1">
+      <c r="D553" s="2">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26362,7 +26388,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="1">
+      <c r="D554" s="2">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26528,7 +26554,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="1">
+      <c r="D559" s="2">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26726,7 +26752,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="1">
+      <c r="D565" s="2">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27346,7 +27372,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="1">
+      <c r="D584" s="2">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (10/09/2026 11:59)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,16 +5159,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5184,7 +5176,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5192,30 +5184,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5515,52 +5489,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5638,7 +5612,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5775,7 +5749,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5912,7 +5886,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5953,7 +5927,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5988,7 +5962,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6029,7 +6003,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6067,7 +6041,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6108,7 +6082,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6149,7 +6123,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6187,7 +6161,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6228,7 +6202,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6269,7 +6243,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6310,7 +6284,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6351,7 +6325,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6453,7 +6427,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6494,7 +6468,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6535,7 +6509,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6576,7 +6550,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6617,7 +6591,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6658,7 +6632,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6731,7 +6705,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6804,7 +6778,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6845,7 +6819,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6886,7 +6860,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6927,7 +6901,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -7000,7 +6974,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7105,7 +7079,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7146,7 +7120,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7187,7 +7161,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7228,7 +7202,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7269,7 +7243,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7310,7 +7284,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7348,7 +7322,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7389,7 +7363,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7430,7 +7404,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7503,7 +7477,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7544,7 +7518,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7617,7 +7591,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7690,7 +7664,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7763,7 +7737,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7833,7 +7807,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7906,7 +7880,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7941,7 +7915,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7982,7 +7956,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8023,7 +7997,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8064,7 +8038,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8105,7 +8079,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8146,7 +8120,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8187,7 +8161,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8228,7 +8202,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8263,7 +8237,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8304,7 +8278,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8342,7 +8316,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8380,7 +8354,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8418,7 +8392,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8456,7 +8430,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8497,7 +8471,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8538,7 +8512,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8579,7 +8553,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8620,7 +8594,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8661,7 +8635,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8702,7 +8676,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8743,7 +8717,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8784,7 +8758,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8863,7 +8837,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8904,7 +8878,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8945,7 +8919,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8986,7 +8960,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9027,7 +9001,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9068,7 +9042,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9109,7 +9083,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9150,7 +9124,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9223,7 +9197,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9264,7 +9238,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9305,7 +9279,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9346,7 +9320,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9387,7 +9361,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9425,7 +9399,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9495,7 +9469,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9536,7 +9510,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9577,7 +9551,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9618,7 +9592,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9720,7 +9694,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9761,7 +9735,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9802,7 +9776,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9843,7 +9817,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9881,7 +9855,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9919,7 +9893,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9960,7 +9934,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -10001,7 +9975,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10042,7 +10016,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10083,7 +10057,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10124,7 +10098,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10165,7 +10139,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10206,7 +10180,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10247,7 +10221,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10285,7 +10259,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10326,7 +10300,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10367,7 +10341,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10437,7 +10411,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10510,7 +10484,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10551,7 +10525,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10592,7 +10566,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10665,7 +10639,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10706,7 +10680,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10747,7 +10721,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10785,7 +10759,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10858,7 +10832,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10896,7 +10870,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10966,7 +10940,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11071,7 +11045,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11112,7 +11086,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11153,7 +11127,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11194,7 +11168,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11235,7 +11209,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11276,7 +11250,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11317,7 +11291,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11390,7 +11364,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11431,7 +11405,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11472,7 +11446,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11513,7 +11487,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11583,7 +11557,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11624,7 +11598,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11665,7 +11639,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11706,7 +11680,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11747,7 +11721,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11788,7 +11762,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11826,7 +11800,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11899,7 +11873,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11940,7 +11914,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11978,7 +11952,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12013,7 +11987,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12054,7 +12028,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12095,7 +12069,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12174,7 +12148,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12215,7 +12189,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12256,7 +12230,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12297,7 +12271,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12338,7 +12312,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12379,7 +12353,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12420,7 +12394,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12461,7 +12435,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12534,7 +12508,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12601,7 +12575,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12674,7 +12648,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12715,7 +12689,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12756,7 +12730,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12797,7 +12771,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12838,7 +12812,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12879,7 +12853,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12952,7 +12926,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12993,7 +12967,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13034,7 +13008,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13075,7 +13049,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13116,7 +13090,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13157,7 +13131,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13195,7 +13169,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13236,7 +13210,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13315,7 +13289,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13356,7 +13330,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13397,7 +13371,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13438,7 +13412,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13476,7 +13450,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13517,7 +13491,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13558,7 +13532,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13596,7 +13570,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13637,7 +13611,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13678,7 +13652,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13719,7 +13693,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13833,7 +13807,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13874,7 +13848,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13915,7 +13889,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13956,7 +13930,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13997,7 +13971,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14358,7 +14332,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14399,7 +14373,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14440,7 +14414,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14481,7 +14455,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14522,7 +14496,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14563,7 +14537,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14604,7 +14578,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14741,7 +14715,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14782,7 +14756,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14855,7 +14829,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14896,7 +14870,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14934,7 +14908,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14972,7 +14946,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15234,7 +15208,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15339,7 +15313,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15380,7 +15354,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15421,7 +15395,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15462,7 +15436,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15500,7 +15474,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15541,7 +15515,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15582,7 +15556,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15623,7 +15597,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15667,7 +15641,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15708,7 +15682,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15749,7 +15723,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15790,7 +15764,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15831,7 +15805,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15875,7 +15849,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15910,7 +15884,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15948,7 +15922,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15983,7 +15957,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16024,7 +15998,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16062,7 +16036,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16103,7 +16077,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16141,7 +16115,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16179,7 +16153,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16217,7 +16191,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16255,7 +16229,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16296,7 +16270,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16334,7 +16308,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16375,7 +16349,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16416,7 +16390,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16521,7 +16495,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16562,7 +16536,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16603,7 +16577,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16644,7 +16618,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16685,7 +16659,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16726,7 +16700,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16767,7 +16741,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16808,7 +16782,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16849,7 +16823,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16884,7 +16858,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16919,7 +16893,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16954,7 +16928,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17027,7 +17001,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17068,7 +17042,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17109,7 +17083,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17150,7 +17124,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17188,7 +17162,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17229,7 +17203,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17270,7 +17244,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17311,7 +17285,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17352,7 +17326,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17393,7 +17367,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17434,7 +17408,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17475,7 +17449,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17516,7 +17490,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17551,7 +17525,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17592,7 +17566,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17633,7 +17607,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17674,7 +17648,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17715,7 +17689,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17756,7 +17730,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17797,7 +17771,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17838,7 +17812,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17943,7 +17917,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17984,7 +17958,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18121,7 +18095,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18191,7 +18165,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18232,7 +18206,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18264,7 +18238,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18305,7 +18279,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18343,7 +18317,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18381,7 +18355,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18419,7 +18393,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18454,7 +18428,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18492,7 +18466,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18530,7 +18504,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18568,7 +18542,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18606,7 +18580,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18644,7 +18618,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18682,7 +18656,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18720,7 +18694,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18761,7 +18735,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18866,7 +18840,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18971,7 +18945,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19009,7 +18983,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19079,7 +19053,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19114,7 +19088,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19152,7 +19126,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19196,7 +19170,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19231,7 +19205,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19269,7 +19243,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19345,7 +19319,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19383,7 +19357,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19453,7 +19427,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19494,7 +19468,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19532,7 +19506,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19570,7 +19544,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19614,7 +19588,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19652,7 +19626,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19693,7 +19667,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19734,7 +19708,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19775,7 +19749,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19941,7 +19915,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19982,7 +19956,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20023,7 +19997,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20064,7 +20038,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20105,7 +20079,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20146,7 +20120,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20187,7 +20161,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20228,7 +20202,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20269,7 +20243,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20342,7 +20316,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20572,7 +20546,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20613,7 +20587,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20654,7 +20628,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20727,7 +20701,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20765,7 +20739,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20803,7 +20777,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20870,7 +20844,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20943,7 +20917,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20984,7 +20958,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21025,7 +20999,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21066,7 +21040,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21133,7 +21107,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21174,7 +21148,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21212,7 +21186,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21250,7 +21224,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21285,7 +21259,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21422,7 +21396,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21457,7 +21431,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21492,7 +21466,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21559,7 +21533,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21600,7 +21574,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21641,7 +21615,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21682,7 +21656,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21720,7 +21694,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21761,7 +21735,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21802,7 +21776,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -22000,7 +21974,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22041,7 +22015,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22172,7 +22146,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22213,7 +22187,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22254,7 +22228,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22295,7 +22269,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22333,7 +22307,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22374,7 +22348,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22415,7 +22389,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22450,7 +22424,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22485,7 +22459,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22552,7 +22526,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22593,7 +22567,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22628,7 +22602,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22663,7 +22637,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22736,7 +22710,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22777,7 +22751,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22815,7 +22789,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22850,7 +22824,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22949,7 +22923,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22993,7 +22967,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23060,7 +23034,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23159,7 +23133,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23200,7 +23174,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23241,7 +23215,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23282,7 +23256,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23320,7 +23294,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23358,7 +23332,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23396,7 +23370,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23437,7 +23411,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23475,7 +23449,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23513,7 +23487,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23551,7 +23525,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23624,7 +23598,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23796,7 +23770,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23837,7 +23811,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23878,7 +23852,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24143,7 +24117,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24184,7 +24158,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24289,7 +24263,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24333,7 +24307,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24374,7 +24348,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24412,7 +24386,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24488,7 +24462,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24532,7 +24506,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24573,7 +24547,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24678,7 +24652,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24722,7 +24696,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24798,7 +24772,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24833,7 +24807,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24874,7 +24848,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24909,7 +24883,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24950,7 +24924,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24991,7 +24965,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25032,7 +25006,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25073,7 +25047,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25178,7 +25152,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25312,7 +25286,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25449,7 +25423,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25586,7 +25560,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25691,7 +25665,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25729,7 +25703,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25930,7 +25904,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25974,7 +25948,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26009,7 +25983,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26044,7 +26018,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26242,7 +26216,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26347,7 +26321,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26388,7 +26362,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26554,7 +26528,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26752,7 +26726,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27372,7 +27346,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>